<commit_message>
Daily TALT data update 2025-09-01
</commit_message>
<xml_diff>
--- a/data/talt_cyano/talt_cyano_digitized.xlsx
+++ b/data/talt_cyano/talt_cyano_digitized.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29212"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29225"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="20435" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ED0097AE-E8BF-4194-85E9-A632FE632A20}"/>
+  <xr:revisionPtr revIDLastSave="20831" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CE9692C1-B11D-466F-9214-9CC4539DAEFC}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1854" uniqueCount="390">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1878" uniqueCount="393">
   <si>
     <t>Date</t>
   </si>
@@ -1197,10 +1197,19 @@
     <t xml:space="preserve">18/08/2025 </t>
   </si>
   <si>
+    <t xml:space="preserve">0.34	</t>
+  </si>
+  <si>
     <t xml:space="preserve">20/08/2025 </t>
   </si>
   <si>
     <t xml:space="preserve">22/08/2025 </t>
+  </si>
+  <si>
+    <t>25/08/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">29/08/2025 </t>
   </si>
 </sst>
 </file>
@@ -1758,7 +1767,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S2707"/>
+  <dimension ref="A1:S2769"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="11.7109375" customWidth="1"/>
@@ -68701,6 +68710,9 @@
       <c r="A2615" t="s">
         <v>387</v>
       </c>
+      <c r="B2615" s="1">
+        <v>0.43541666666666667</v>
+      </c>
       <c r="C2615" s="3" t="s">
         <v>20</v>
       </c>
@@ -68719,6 +68731,18 @@
       <c r="H2615">
         <v>0</v>
       </c>
+      <c r="L2615">
+        <v>11.3</v>
+      </c>
+      <c r="M2615">
+        <v>98.4</v>
+      </c>
+      <c r="N2615">
+        <v>1.01</v>
+      </c>
+      <c r="O2615" t="s">
+        <v>388</v>
+      </c>
       <c r="P2615" t="s">
         <v>319</v>
       </c>
@@ -68752,6 +68776,9 @@
       </c>
     </row>
     <row r="2618" spans="1:18">
+      <c r="B2618" s="1">
+        <v>0.45694444444444443</v>
+      </c>
       <c r="C2618" s="3" t="s">
         <v>25</v>
       </c>
@@ -68767,6 +68794,18 @@
       <c r="H2618">
         <v>0</v>
       </c>
+      <c r="L2618">
+        <v>12.6</v>
+      </c>
+      <c r="M2618">
+        <v>88.4</v>
+      </c>
+      <c r="N2618">
+        <v>2.84</v>
+      </c>
+      <c r="O2618">
+        <v>0.17</v>
+      </c>
     </row>
     <row r="2619" spans="1:18">
       <c r="D2619">
@@ -68797,6 +68836,9 @@
       </c>
     </row>
     <row r="2621" spans="1:18">
+      <c r="B2621" s="1">
+        <v>0.47430555555555554</v>
+      </c>
       <c r="C2621" s="3" t="s">
         <v>27</v>
       </c>
@@ -68812,6 +68854,18 @@
       <c r="H2621">
         <v>0.09</v>
       </c>
+      <c r="L2621">
+        <v>11.3</v>
+      </c>
+      <c r="M2621">
+        <v>99</v>
+      </c>
+      <c r="N2621">
+        <v>2.12</v>
+      </c>
+      <c r="O2621">
+        <v>0.22</v>
+      </c>
     </row>
     <row r="2622" spans="1:18">
       <c r="D2622">
@@ -68842,6 +68896,9 @@
       </c>
     </row>
     <row r="2624" spans="1:18">
+      <c r="B2624" s="1">
+        <v>0.49236111111111114</v>
+      </c>
       <c r="C2624" s="3" t="s">
         <v>58</v>
       </c>
@@ -68857,8 +68914,20 @@
       <c r="H2624">
         <v>2</v>
       </c>
-    </row>
-    <row r="2625" spans="3:8">
+      <c r="L2624">
+        <v>11.7</v>
+      </c>
+      <c r="M2624">
+        <v>90.6</v>
+      </c>
+      <c r="N2624">
+        <v>7.08</v>
+      </c>
+      <c r="O2624">
+        <v>4.43</v>
+      </c>
+    </row>
+    <row r="2625" spans="2:15">
       <c r="D2625">
         <v>2</v>
       </c>
@@ -68872,7 +68941,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2626" spans="3:8">
+    <row r="2626" spans="2:15">
       <c r="D2626">
         <v>3</v>
       </c>
@@ -68886,7 +68955,10 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="2627" spans="3:8">
+    <row r="2627" spans="2:15">
+      <c r="B2627" s="1">
+        <v>0.50694444444444442</v>
+      </c>
       <c r="C2627" s="3" t="s">
         <v>29</v>
       </c>
@@ -68902,8 +68974,20 @@
       <c r="H2627">
         <v>0</v>
       </c>
-    </row>
-    <row r="2628" spans="3:8">
+      <c r="L2627">
+        <v>11.8</v>
+      </c>
+      <c r="M2627">
+        <v>111.2</v>
+      </c>
+      <c r="N2627">
+        <v>0.86</v>
+      </c>
+      <c r="O2627">
+        <v>0.17</v>
+      </c>
+    </row>
+    <row r="2628" spans="2:15">
       <c r="D2628">
         <v>2</v>
       </c>
@@ -68917,7 +69001,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2629" spans="3:8">
+    <row r="2629" spans="2:15">
       <c r="D2629">
         <v>3</v>
       </c>
@@ -68931,7 +69015,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2630" spans="3:8">
+    <row r="2630" spans="2:15">
+      <c r="B2630" s="1">
+        <v>0.51597222222222228</v>
+      </c>
       <c r="C2630" s="3" t="s">
         <v>30</v>
       </c>
@@ -68947,8 +69034,20 @@
       <c r="H2630">
         <v>0</v>
       </c>
-    </row>
-    <row r="2631" spans="3:8">
+      <c r="L2630">
+        <v>11.9</v>
+      </c>
+      <c r="M2630">
+        <v>105</v>
+      </c>
+      <c r="N2630">
+        <v>0.54</v>
+      </c>
+      <c r="O2630">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="2631" spans="2:15">
       <c r="D2631">
         <v>2</v>
       </c>
@@ -68962,7 +69061,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2632" spans="3:8">
+    <row r="2632" spans="2:15">
       <c r="D2632">
         <v>3</v>
       </c>
@@ -68976,7 +69075,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2633" spans="3:8">
+    <row r="2633" spans="2:15">
+      <c r="B2633" s="1">
+        <v>0.52916666666666667</v>
+      </c>
       <c r="C2633" s="3" t="s">
         <v>31</v>
       </c>
@@ -68992,8 +69094,20 @@
       <c r="H2633">
         <v>0</v>
       </c>
-    </row>
-    <row r="2634" spans="3:8">
+      <c r="L2633">
+        <v>12.3</v>
+      </c>
+      <c r="M2633">
+        <v>102.9</v>
+      </c>
+      <c r="N2633">
+        <v>0.31</v>
+      </c>
+      <c r="O2633">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="2634" spans="2:15">
       <c r="D2634">
         <v>2</v>
       </c>
@@ -69007,7 +69121,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2635" spans="3:8">
+    <row r="2635" spans="2:15">
       <c r="D2635">
         <v>3</v>
       </c>
@@ -69021,7 +69135,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2636" spans="3:8">
+    <row r="2636" spans="2:15">
+      <c r="B2636" s="1">
+        <v>0.54305555555555551</v>
+      </c>
       <c r="C2636" s="3" t="s">
         <v>32</v>
       </c>
@@ -69037,8 +69154,20 @@
       <c r="H2636">
         <v>0.03</v>
       </c>
-    </row>
-    <row r="2637" spans="3:8">
+      <c r="L2636">
+        <v>11.9</v>
+      </c>
+      <c r="M2636">
+        <v>100.4</v>
+      </c>
+      <c r="N2636">
+        <v>0.87</v>
+      </c>
+      <c r="O2636">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="2637" spans="2:15">
       <c r="D2637">
         <v>2</v>
       </c>
@@ -69052,7 +69181,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2638" spans="3:8">
+    <row r="2638" spans="2:15">
       <c r="D2638">
         <v>3</v>
       </c>
@@ -69066,7 +69195,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2639" spans="3:8">
+    <row r="2639" spans="2:15">
+      <c r="B2639" s="1">
+        <v>0.56666666666666665</v>
+      </c>
       <c r="C2639" s="3" t="s">
         <v>41</v>
       </c>
@@ -69082,8 +69214,20 @@
       <c r="H2639">
         <v>0</v>
       </c>
-    </row>
-    <row r="2640" spans="3:8">
+      <c r="L2639">
+        <v>12.5</v>
+      </c>
+      <c r="M2639">
+        <v>103.4</v>
+      </c>
+      <c r="N2639">
+        <v>1.34</v>
+      </c>
+      <c r="O2639">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="2640" spans="2:15">
       <c r="D2640">
         <v>2</v>
       </c>
@@ -69112,6 +69256,9 @@
       </c>
     </row>
     <row r="2642" spans="1:16">
+      <c r="B2642" s="1">
+        <v>0.5756944444444444</v>
+      </c>
       <c r="C2642" s="3" t="s">
         <v>34</v>
       </c>
@@ -69126,6 +69273,18 @@
       </c>
       <c r="H2642">
         <v>0</v>
+      </c>
+      <c r="L2642">
+        <v>13.2</v>
+      </c>
+      <c r="M2642">
+        <v>94.1</v>
+      </c>
+      <c r="N2642">
+        <v>2.4700000000000002</v>
+      </c>
+      <c r="O2642">
+        <v>0.27</v>
       </c>
     </row>
     <row r="2643" spans="1:16">
@@ -69162,7 +69321,10 @@
     </row>
     <row r="2646" spans="1:16">
       <c r="A2646" t="s">
-        <v>388</v>
+        <v>389</v>
+      </c>
+      <c r="B2646" s="1">
+        <v>0.48958333333333331</v>
       </c>
       <c r="C2646" s="3" t="s">
         <v>20</v>
@@ -69182,6 +69344,18 @@
       <c r="H2646">
         <v>0</v>
       </c>
+      <c r="L2646">
+        <v>10.8</v>
+      </c>
+      <c r="M2646">
+        <v>90.6</v>
+      </c>
+      <c r="N2646">
+        <v>4.1500000000000004</v>
+      </c>
+      <c r="O2646">
+        <v>0.08</v>
+      </c>
       <c r="P2646" t="s">
         <v>147</v>
       </c>
@@ -69215,6 +69389,9 @@
       </c>
     </row>
     <row r="2649" spans="1:16">
+      <c r="B2649" s="1">
+        <v>0.50069444444444444</v>
+      </c>
       <c r="C2649" s="3" t="s">
         <v>25</v>
       </c>
@@ -69230,6 +69407,18 @@
       <c r="H2649">
         <v>0</v>
       </c>
+      <c r="L2649">
+        <v>10.8</v>
+      </c>
+      <c r="M2649">
+        <v>95.8</v>
+      </c>
+      <c r="N2649">
+        <v>4.93</v>
+      </c>
+      <c r="O2649">
+        <v>0.15</v>
+      </c>
     </row>
     <row r="2650" spans="1:16">
       <c r="D2650">
@@ -69260,6 +69449,9 @@
       </c>
     </row>
     <row r="2652" spans="1:16">
+      <c r="B2652" s="1">
+        <v>0.51597222222222228</v>
+      </c>
       <c r="C2652" s="3" t="s">
         <v>27</v>
       </c>
@@ -69275,6 +69467,18 @@
       <c r="H2652">
         <v>0</v>
       </c>
+      <c r="L2652">
+        <v>9.9</v>
+      </c>
+      <c r="M2652">
+        <v>97.1</v>
+      </c>
+      <c r="N2652">
+        <v>10.51</v>
+      </c>
+      <c r="O2652">
+        <v>0.28000000000000003</v>
+      </c>
     </row>
     <row r="2653" spans="1:16">
       <c r="D2653">
@@ -69305,6 +69509,9 @@
       </c>
     </row>
     <row r="2655" spans="1:16">
+      <c r="B2655" s="1">
+        <v>0.52569444444444446</v>
+      </c>
       <c r="C2655" s="3" t="s">
         <v>58</v>
       </c>
@@ -69320,6 +69527,18 @@
       <c r="H2655">
         <v>0.15</v>
       </c>
+      <c r="L2655">
+        <v>9.3000000000000007</v>
+      </c>
+      <c r="M2655">
+        <v>99.3</v>
+      </c>
+      <c r="N2655">
+        <v>13.22</v>
+      </c>
+      <c r="O2655">
+        <v>0.91</v>
+      </c>
     </row>
     <row r="2656" spans="1:16">
       <c r="D2656">
@@ -69335,7 +69554,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2657" spans="3:8">
+    <row r="2657" spans="2:15">
       <c r="D2657">
         <v>3</v>
       </c>
@@ -69349,7 +69568,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2658" spans="3:8">
+    <row r="2658" spans="2:15">
+      <c r="B2658" s="1">
+        <v>0.53611111111111109</v>
+      </c>
       <c r="C2658" s="3" t="s">
         <v>29</v>
       </c>
@@ -69365,8 +69587,20 @@
       <c r="H2658">
         <v>7.0000000000000007E-2</v>
       </c>
-    </row>
-    <row r="2659" spans="3:8">
+      <c r="L2658">
+        <v>9.3000000000000007</v>
+      </c>
+      <c r="M2658">
+        <v>101.3</v>
+      </c>
+      <c r="N2658">
+        <v>15.49</v>
+      </c>
+      <c r="O2658">
+        <v>2.31</v>
+      </c>
+    </row>
+    <row r="2659" spans="2:15">
       <c r="D2659">
         <v>2</v>
       </c>
@@ -69380,7 +69614,7 @@
         <v>0.08</v>
       </c>
     </row>
-    <row r="2660" spans="3:8">
+    <row r="2660" spans="2:15">
       <c r="D2660">
         <v>3</v>
       </c>
@@ -69394,7 +69628,10 @@
         <v>0.08</v>
       </c>
     </row>
-    <row r="2661" spans="3:8">
+    <row r="2661" spans="2:15">
+      <c r="B2661" s="1">
+        <v>0.54652777777777772</v>
+      </c>
       <c r="C2661" s="3" t="s">
         <v>30</v>
       </c>
@@ -69410,8 +69647,20 @@
       <c r="H2661">
         <v>18.75</v>
       </c>
-    </row>
-    <row r="2662" spans="3:8">
+      <c r="L2661">
+        <v>9.3000000000000007</v>
+      </c>
+      <c r="M2661">
+        <v>96.7</v>
+      </c>
+      <c r="N2661">
+        <v>20.260000000000002</v>
+      </c>
+      <c r="O2661">
+        <v>3.07</v>
+      </c>
+    </row>
+    <row r="2662" spans="2:15">
       <c r="D2662">
         <v>2</v>
       </c>
@@ -69425,7 +69674,7 @@
         <v>9.0500000000000007</v>
       </c>
     </row>
-    <row r="2663" spans="3:8">
+    <row r="2663" spans="2:15">
       <c r="D2663">
         <v>3</v>
       </c>
@@ -69439,7 +69688,10 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="2664" spans="3:8">
+    <row r="2664" spans="2:15">
+      <c r="B2664" s="1">
+        <v>0.5541666666666667</v>
+      </c>
       <c r="C2664" s="3" t="s">
         <v>31</v>
       </c>
@@ -69455,8 +69707,20 @@
       <c r="H2664">
         <v>0</v>
       </c>
-    </row>
-    <row r="2665" spans="3:8">
+      <c r="L2664">
+        <v>12.6</v>
+      </c>
+      <c r="M2664">
+        <v>102.8</v>
+      </c>
+      <c r="N2664">
+        <v>3.31</v>
+      </c>
+      <c r="O2664">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="2665" spans="2:15">
       <c r="D2665">
         <v>2</v>
       </c>
@@ -69470,7 +69734,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2666" spans="3:8">
+    <row r="2666" spans="2:15">
       <c r="D2666">
         <v>3</v>
       </c>
@@ -69484,7 +69748,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2667" spans="3:8">
+    <row r="2667" spans="2:15">
+      <c r="B2667" s="1">
+        <v>0.56111111111111112</v>
+      </c>
       <c r="C2667" s="3" t="s">
         <v>32</v>
       </c>
@@ -69500,8 +69767,20 @@
       <c r="H2667">
         <v>0</v>
       </c>
-    </row>
-    <row r="2668" spans="3:8">
+      <c r="L2667">
+        <v>10.4</v>
+      </c>
+      <c r="M2667">
+        <v>98.8</v>
+      </c>
+      <c r="N2667">
+        <v>9.1199999999999992</v>
+      </c>
+      <c r="O2667">
+        <v>0.32</v>
+      </c>
+    </row>
+    <row r="2668" spans="2:15">
       <c r="D2668">
         <v>2</v>
       </c>
@@ -69515,7 +69794,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2669" spans="3:8">
+    <row r="2669" spans="2:15">
       <c r="D2669">
         <v>3</v>
       </c>
@@ -69529,7 +69808,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2670" spans="3:8">
+    <row r="2670" spans="2:15">
+      <c r="B2670" s="1">
+        <v>0.57708333333333328</v>
+      </c>
       <c r="C2670" s="3" t="s">
         <v>41</v>
       </c>
@@ -69545,8 +69827,20 @@
       <c r="H2670">
         <v>0</v>
       </c>
-    </row>
-    <row r="2671" spans="3:8">
+      <c r="L2670">
+        <v>11.5</v>
+      </c>
+      <c r="M2670">
+        <v>105.1</v>
+      </c>
+      <c r="N2670">
+        <v>1.66</v>
+      </c>
+      <c r="O2670">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="2671" spans="2:15">
       <c r="D2671">
         <v>2</v>
       </c>
@@ -69560,7 +69854,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2672" spans="3:8">
+    <row r="2672" spans="2:15">
       <c r="D2672">
         <v>3</v>
       </c>
@@ -69575,6 +69869,9 @@
       </c>
     </row>
     <row r="2673" spans="1:16">
+      <c r="B2673" s="1">
+        <v>0.58333333333333337</v>
+      </c>
       <c r="C2673" s="3" t="s">
         <v>34</v>
       </c>
@@ -69589,6 +69886,18 @@
       </c>
       <c r="H2673">
         <v>0</v>
+      </c>
+      <c r="L2673">
+        <v>11</v>
+      </c>
+      <c r="M2673">
+        <v>96.6</v>
+      </c>
+      <c r="N2673">
+        <v>1.94</v>
+      </c>
+      <c r="O2673">
+        <v>0.04</v>
       </c>
     </row>
     <row r="2674" spans="1:16">
@@ -69625,7 +69934,10 @@
     </row>
     <row r="2677" spans="1:16">
       <c r="A2677" t="s">
-        <v>389</v>
+        <v>390</v>
+      </c>
+      <c r="B2677" s="1">
+        <v>0.50069444444444444</v>
       </c>
       <c r="C2677" s="3" t="s">
         <v>20</v>
@@ -69645,6 +69957,18 @@
       <c r="H2677">
         <v>0</v>
       </c>
+      <c r="L2677">
+        <v>12.2</v>
+      </c>
+      <c r="M2677">
+        <v>95.7</v>
+      </c>
+      <c r="N2677">
+        <v>1.1399999999999999</v>
+      </c>
+      <c r="O2677">
+        <v>0.08</v>
+      </c>
       <c r="P2677" t="s">
         <v>157</v>
       </c>
@@ -69678,6 +70002,9 @@
       </c>
     </row>
     <row r="2680" spans="1:16">
+      <c r="B2680" s="1">
+        <v>0.5180555555555556</v>
+      </c>
       <c r="C2680" s="3" t="s">
         <v>25</v>
       </c>
@@ -69693,6 +70020,18 @@
       <c r="H2680">
         <v>0</v>
       </c>
+      <c r="L2680">
+        <v>11.3</v>
+      </c>
+      <c r="M2680">
+        <v>100.3</v>
+      </c>
+      <c r="N2680">
+        <v>1.94</v>
+      </c>
+      <c r="O2680">
+        <v>0.15</v>
+      </c>
     </row>
     <row r="2681" spans="1:16">
       <c r="D2681">
@@ -69723,6 +70062,9 @@
       </c>
     </row>
     <row r="2683" spans="1:16">
+      <c r="B2683" s="1">
+        <v>0.57152777777777775</v>
+      </c>
       <c r="C2683" s="3" t="s">
         <v>27</v>
       </c>
@@ -69738,6 +70080,18 @@
       <c r="H2683">
         <v>0</v>
       </c>
+      <c r="L2683">
+        <v>11.5</v>
+      </c>
+      <c r="M2683">
+        <v>92.8</v>
+      </c>
+      <c r="N2683">
+        <v>1.75</v>
+      </c>
+      <c r="O2683">
+        <v>0.06</v>
+      </c>
     </row>
     <row r="2684" spans="1:16">
       <c r="D2684">
@@ -69768,6 +70122,9 @@
       </c>
     </row>
     <row r="2686" spans="1:16">
+      <c r="B2686" s="1">
+        <v>0.58958333333333335</v>
+      </c>
       <c r="C2686" s="3" t="s">
         <v>58</v>
       </c>
@@ -69783,6 +70140,18 @@
       <c r="H2686">
         <v>0</v>
       </c>
+      <c r="L2686">
+        <v>10.9</v>
+      </c>
+      <c r="M2686">
+        <v>102.5</v>
+      </c>
+      <c r="N2686">
+        <v>1.41</v>
+      </c>
+      <c r="O2686">
+        <v>0.05</v>
+      </c>
     </row>
     <row r="2687" spans="1:16">
       <c r="D2687">
@@ -69812,7 +70181,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2689" spans="3:8">
+    <row r="2689" spans="2:15">
+      <c r="B2689" s="1">
+        <v>0.61319444444444449</v>
+      </c>
       <c r="C2689" s="3" t="s">
         <v>29</v>
       </c>
@@ -69828,8 +70200,20 @@
       <c r="H2689">
         <v>0</v>
       </c>
-    </row>
-    <row r="2690" spans="3:8">
+      <c r="L2689">
+        <v>10.7</v>
+      </c>
+      <c r="M2689">
+        <v>103.6</v>
+      </c>
+      <c r="N2689">
+        <v>4.34</v>
+      </c>
+      <c r="O2689">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="2690" spans="2:15">
       <c r="D2690">
         <v>2</v>
       </c>
@@ -69843,7 +70227,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2691" spans="3:8">
+    <row r="2691" spans="2:15">
       <c r="D2691">
         <v>3</v>
       </c>
@@ -69857,7 +70241,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2692" spans="3:8">
+    <row r="2692" spans="2:15">
+      <c r="B2692" s="1">
+        <v>0.63194444444444442</v>
+      </c>
       <c r="C2692" s="3" t="s">
         <v>30</v>
       </c>
@@ -69873,8 +70260,20 @@
       <c r="H2692">
         <v>0.28000000000000003</v>
       </c>
-    </row>
-    <row r="2693" spans="3:8">
+      <c r="L2692">
+        <v>11</v>
+      </c>
+      <c r="M2692">
+        <v>104.3</v>
+      </c>
+      <c r="N2692">
+        <v>2.39</v>
+      </c>
+      <c r="O2692">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="2693" spans="2:15">
       <c r="D2693">
         <v>2</v>
       </c>
@@ -69888,7 +70287,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2694" spans="3:8">
+    <row r="2694" spans="2:15">
       <c r="D2694">
         <v>3</v>
       </c>
@@ -69902,7 +70301,10 @@
         <v>13.18</v>
       </c>
     </row>
-    <row r="2695" spans="3:8">
+    <row r="2695" spans="2:15">
+      <c r="B2695" s="1">
+        <v>0.64513888888888893</v>
+      </c>
       <c r="C2695" s="3" t="s">
         <v>31</v>
       </c>
@@ -69918,8 +70320,20 @@
       <c r="H2695">
         <v>0</v>
       </c>
-    </row>
-    <row r="2696" spans="3:8">
+      <c r="L2695">
+        <v>12</v>
+      </c>
+      <c r="M2695">
+        <v>101.6</v>
+      </c>
+      <c r="N2695">
+        <v>1.49</v>
+      </c>
+      <c r="O2695">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="2696" spans="2:15">
       <c r="D2696">
         <v>2</v>
       </c>
@@ -69933,7 +70347,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2697" spans="3:8">
+    <row r="2697" spans="2:15">
       <c r="D2697">
         <v>3</v>
       </c>
@@ -69947,7 +70361,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2698" spans="3:8">
+    <row r="2698" spans="2:15">
+      <c r="B2698" s="1">
+        <v>0.65833333333333333</v>
+      </c>
       <c r="C2698" s="3" t="s">
         <v>32</v>
       </c>
@@ -69963,8 +70380,20 @@
       <c r="H2698">
         <v>0</v>
       </c>
-    </row>
-    <row r="2699" spans="3:8">
+      <c r="L2698">
+        <v>11.6</v>
+      </c>
+      <c r="M2698">
+        <v>105.6</v>
+      </c>
+      <c r="N2698">
+        <v>1.98</v>
+      </c>
+      <c r="O2698">
+        <v>0.19</v>
+      </c>
+    </row>
+    <row r="2699" spans="2:15">
       <c r="D2699">
         <v>2</v>
       </c>
@@ -69978,7 +70407,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2700" spans="3:8">
+    <row r="2700" spans="2:15">
       <c r="D2700">
         <v>3</v>
       </c>
@@ -69992,7 +70421,10 @@
         <v>0.28000000000000003</v>
       </c>
     </row>
-    <row r="2701" spans="3:8">
+    <row r="2701" spans="2:15">
+      <c r="B2701" s="1">
+        <v>0.67222222222222228</v>
+      </c>
       <c r="C2701" s="3" t="s">
         <v>41</v>
       </c>
@@ -70008,8 +70440,20 @@
       <c r="H2701">
         <v>0.04</v>
       </c>
-    </row>
-    <row r="2702" spans="3:8">
+      <c r="L2701">
+        <v>12.6</v>
+      </c>
+      <c r="M2701">
+        <v>105.8</v>
+      </c>
+      <c r="N2701">
+        <v>6.63</v>
+      </c>
+      <c r="O2701">
+        <v>0.92</v>
+      </c>
+    </row>
+    <row r="2702" spans="2:15">
       <c r="D2702">
         <v>2</v>
       </c>
@@ -70023,7 +70467,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="2703" spans="3:8">
+    <row r="2703" spans="2:15">
       <c r="D2703">
         <v>3</v>
       </c>
@@ -70037,7 +70481,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="2704" spans="3:8">
+    <row r="2704" spans="2:15">
       <c r="C2704" s="3" t="s">
         <v>34</v>
       </c>
@@ -70053,8 +70497,20 @@
       <c r="H2704">
         <v>0</v>
       </c>
-    </row>
-    <row r="2705" spans="3:8">
+      <c r="L2704">
+        <v>14.3</v>
+      </c>
+      <c r="M2704">
+        <v>106.6</v>
+      </c>
+      <c r="N2704">
+        <v>9.81</v>
+      </c>
+      <c r="O2704">
+        <v>0.82</v>
+      </c>
+    </row>
+    <row r="2705" spans="1:15">
       <c r="C2705" s="3"/>
       <c r="D2705">
         <v>2</v>
@@ -70069,7 +70525,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2706" spans="3:8">
+    <row r="2706" spans="1:15">
       <c r="D2706">
         <v>3</v>
       </c>
@@ -70083,8 +70539,1225 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2707" spans="3:8" s="19" customFormat="1">
+    <row r="2707" spans="1:15" s="19" customFormat="1">
       <c r="E2707" s="36"/>
+    </row>
+    <row r="2708" spans="1:15">
+      <c r="A2708" t="s">
+        <v>391</v>
+      </c>
+      <c r="B2708" s="1">
+        <v>0.55833333333333335</v>
+      </c>
+      <c r="C2708" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2708">
+        <v>1</v>
+      </c>
+      <c r="E2708" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F2708">
+        <v>0.1</v>
+      </c>
+      <c r="G2708">
+        <v>0</v>
+      </c>
+      <c r="H2708">
+        <v>0</v>
+      </c>
+      <c r="L2708">
+        <v>12.5</v>
+      </c>
+      <c r="M2708">
+        <v>97.5</v>
+      </c>
+      <c r="N2708">
+        <v>0.98</v>
+      </c>
+      <c r="O2708">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="2709" spans="1:15">
+      <c r="D2709">
+        <v>2</v>
+      </c>
+      <c r="F2709">
+        <v>0.1</v>
+      </c>
+      <c r="G2709">
+        <v>0</v>
+      </c>
+      <c r="H2709">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2710" spans="1:15">
+      <c r="D2710">
+        <v>3</v>
+      </c>
+      <c r="F2710">
+        <v>0.1</v>
+      </c>
+      <c r="G2710">
+        <v>0</v>
+      </c>
+      <c r="H2710">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2711" spans="1:15">
+      <c r="B2711" s="1">
+        <v>0.57013888888888886</v>
+      </c>
+      <c r="C2711" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2711">
+        <v>1</v>
+      </c>
+      <c r="F2711">
+        <v>0.1</v>
+      </c>
+      <c r="G2711">
+        <v>0</v>
+      </c>
+      <c r="H2711">
+        <v>0</v>
+      </c>
+      <c r="L2711">
+        <v>11.7</v>
+      </c>
+      <c r="M2711">
+        <v>95.2</v>
+      </c>
+      <c r="N2711">
+        <v>3.69</v>
+      </c>
+      <c r="O2711">
+        <v>0.14000000000000001</v>
+      </c>
+    </row>
+    <row r="2712" spans="1:15">
+      <c r="D2712">
+        <v>2</v>
+      </c>
+      <c r="F2712">
+        <v>0.1</v>
+      </c>
+      <c r="G2712">
+        <v>0</v>
+      </c>
+      <c r="H2712">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2713" spans="1:15">
+      <c r="D2713">
+        <v>3</v>
+      </c>
+      <c r="F2713">
+        <v>0.1</v>
+      </c>
+      <c r="G2713">
+        <v>0</v>
+      </c>
+      <c r="H2713">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2714" spans="1:15">
+      <c r="B2714" s="1">
+        <v>0.57986111111111116</v>
+      </c>
+      <c r="C2714" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D2714">
+        <v>1</v>
+      </c>
+      <c r="F2714">
+        <v>0.1</v>
+      </c>
+      <c r="G2714">
+        <v>0</v>
+      </c>
+      <c r="H2714">
+        <v>0</v>
+      </c>
+      <c r="L2714">
+        <v>11.1</v>
+      </c>
+      <c r="M2714">
+        <v>100.1</v>
+      </c>
+      <c r="N2714">
+        <v>0.76</v>
+      </c>
+      <c r="O2714">
+        <v>0.44</v>
+      </c>
+    </row>
+    <row r="2715" spans="1:15">
+      <c r="D2715">
+        <v>2</v>
+      </c>
+      <c r="F2715">
+        <v>0.1</v>
+      </c>
+      <c r="G2715">
+        <v>0</v>
+      </c>
+      <c r="H2715">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2716" spans="1:15">
+      <c r="D2716">
+        <v>3</v>
+      </c>
+      <c r="F2716">
+        <v>0.1</v>
+      </c>
+      <c r="G2716">
+        <v>0</v>
+      </c>
+      <c r="H2716">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2717" spans="1:15">
+      <c r="B2717" s="1">
+        <v>0.59097222222222223</v>
+      </c>
+      <c r="C2717" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D2717">
+        <v>1</v>
+      </c>
+      <c r="F2717">
+        <v>0.1</v>
+      </c>
+      <c r="G2717">
+        <v>0</v>
+      </c>
+      <c r="H2717">
+        <v>0</v>
+      </c>
+      <c r="L2717">
+        <v>11.5</v>
+      </c>
+      <c r="M2717">
+        <v>101.3</v>
+      </c>
+      <c r="N2717">
+        <v>0.64</v>
+      </c>
+      <c r="O2717">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="2718" spans="1:15">
+      <c r="D2718">
+        <v>2</v>
+      </c>
+      <c r="F2718">
+        <v>0.1</v>
+      </c>
+      <c r="G2718">
+        <v>0</v>
+      </c>
+      <c r="H2718">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2719" spans="1:15">
+      <c r="D2719">
+        <v>3</v>
+      </c>
+      <c r="F2719">
+        <v>0.1</v>
+      </c>
+      <c r="G2719">
+        <v>0</v>
+      </c>
+      <c r="H2719">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2720" spans="1:15">
+      <c r="B2720" s="1">
+        <v>0.60277777777777775</v>
+      </c>
+      <c r="C2720" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D2720">
+        <v>1</v>
+      </c>
+      <c r="F2720">
+        <v>0.1</v>
+      </c>
+      <c r="G2720">
+        <v>0</v>
+      </c>
+      <c r="H2720">
+        <v>0</v>
+      </c>
+      <c r="L2720">
+        <v>11.4</v>
+      </c>
+      <c r="M2720">
+        <v>108.2</v>
+      </c>
+      <c r="N2720">
+        <v>0.68</v>
+      </c>
+      <c r="O2720">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="2721" spans="2:15">
+      <c r="D2721">
+        <v>2</v>
+      </c>
+      <c r="F2721">
+        <v>0.1</v>
+      </c>
+      <c r="G2721">
+        <v>0</v>
+      </c>
+      <c r="H2721">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2722" spans="2:15">
+      <c r="D2722">
+        <v>3</v>
+      </c>
+      <c r="F2722">
+        <v>0.1</v>
+      </c>
+      <c r="G2722">
+        <v>0</v>
+      </c>
+      <c r="H2722">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2723" spans="2:15">
+      <c r="B2723" s="1">
+        <v>0.60833333333333328</v>
+      </c>
+      <c r="C2723" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D2723">
+        <v>1</v>
+      </c>
+      <c r="F2723">
+        <v>0.1</v>
+      </c>
+      <c r="G2723">
+        <v>0</v>
+      </c>
+      <c r="H2723">
+        <v>0</v>
+      </c>
+      <c r="L2723">
+        <v>11.3</v>
+      </c>
+      <c r="M2723">
+        <v>103.9</v>
+      </c>
+      <c r="N2723">
+        <v>0.67</v>
+      </c>
+      <c r="O2723">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="2724" spans="2:15">
+      <c r="D2724">
+        <v>2</v>
+      </c>
+      <c r="F2724">
+        <v>0.1</v>
+      </c>
+      <c r="G2724">
+        <v>0</v>
+      </c>
+      <c r="H2724">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2725" spans="2:15">
+      <c r="D2725">
+        <v>3</v>
+      </c>
+      <c r="F2725">
+        <v>0.1</v>
+      </c>
+      <c r="G2725">
+        <v>0</v>
+      </c>
+      <c r="H2725">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2726" spans="2:15">
+      <c r="B2726" s="1">
+        <v>0.61805555555555558</v>
+      </c>
+      <c r="C2726" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D2726">
+        <v>1</v>
+      </c>
+      <c r="F2726">
+        <v>0.1</v>
+      </c>
+      <c r="G2726">
+        <v>0</v>
+      </c>
+      <c r="H2726">
+        <v>0</v>
+      </c>
+      <c r="L2726">
+        <v>12.9</v>
+      </c>
+      <c r="M2726">
+        <v>100.4</v>
+      </c>
+      <c r="N2726">
+        <v>0.23</v>
+      </c>
+      <c r="O2726">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="2727" spans="2:15">
+      <c r="D2727">
+        <v>2</v>
+      </c>
+      <c r="F2727">
+        <v>0.1</v>
+      </c>
+      <c r="G2727">
+        <v>0</v>
+      </c>
+      <c r="H2727">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2728" spans="2:15">
+      <c r="D2728">
+        <v>3</v>
+      </c>
+      <c r="F2728">
+        <v>0.1</v>
+      </c>
+      <c r="G2728">
+        <v>0</v>
+      </c>
+      <c r="H2728">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2729" spans="2:15">
+      <c r="B2729" s="1">
+        <v>0.63402777777777775</v>
+      </c>
+      <c r="C2729" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D2729">
+        <v>1</v>
+      </c>
+      <c r="F2729">
+        <v>0.1</v>
+      </c>
+      <c r="G2729">
+        <v>0</v>
+      </c>
+      <c r="H2729">
+        <v>0</v>
+      </c>
+      <c r="L2729">
+        <v>11.6</v>
+      </c>
+      <c r="M2729">
+        <v>96.7</v>
+      </c>
+      <c r="N2729">
+        <v>1.28</v>
+      </c>
+      <c r="O2729">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="2730" spans="2:15">
+      <c r="D2730">
+        <v>2</v>
+      </c>
+      <c r="F2730">
+        <v>0.1</v>
+      </c>
+      <c r="G2730">
+        <v>0</v>
+      </c>
+      <c r="H2730">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2731" spans="2:15">
+      <c r="D2731">
+        <v>3</v>
+      </c>
+      <c r="F2731">
+        <v>0.1</v>
+      </c>
+      <c r="G2731">
+        <v>0</v>
+      </c>
+      <c r="H2731">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2732" spans="2:15">
+      <c r="B2732" s="1">
+        <v>0.65</v>
+      </c>
+      <c r="C2732" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="D2732">
+        <v>1</v>
+      </c>
+      <c r="F2732">
+        <v>0.1</v>
+      </c>
+      <c r="G2732">
+        <v>10.78</v>
+      </c>
+      <c r="H2732">
+        <v>0</v>
+      </c>
+      <c r="L2732">
+        <v>12.6</v>
+      </c>
+      <c r="M2732">
+        <v>101.4</v>
+      </c>
+      <c r="N2732">
+        <v>3.71</v>
+      </c>
+      <c r="O2732">
+        <v>2.68</v>
+      </c>
+    </row>
+    <row r="2733" spans="2:15">
+      <c r="D2733">
+        <v>2</v>
+      </c>
+      <c r="F2733">
+        <v>0</v>
+      </c>
+      <c r="G2733">
+        <v>9.01</v>
+      </c>
+      <c r="H2733">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="2734" spans="2:15">
+      <c r="D2734">
+        <v>3</v>
+      </c>
+      <c r="F2734">
+        <v>0.1</v>
+      </c>
+      <c r="G2734">
+        <v>3.01</v>
+      </c>
+      <c r="H2734">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="2735" spans="2:15">
+      <c r="B2735" s="1">
+        <v>0.66319444444444442</v>
+      </c>
+      <c r="C2735" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="D2735">
+        <v>1</v>
+      </c>
+      <c r="F2735">
+        <v>0.1</v>
+      </c>
+      <c r="G2735">
+        <v>1.04</v>
+      </c>
+      <c r="H2735">
+        <v>0.09</v>
+      </c>
+      <c r="L2735">
+        <v>13.9</v>
+      </c>
+      <c r="M2735">
+        <v>98.9</v>
+      </c>
+      <c r="N2735">
+        <v>2.31</v>
+      </c>
+      <c r="O2735">
+        <v>1.69</v>
+      </c>
+    </row>
+    <row r="2736" spans="2:15">
+      <c r="C2736" s="3"/>
+      <c r="D2736">
+        <v>2</v>
+      </c>
+      <c r="F2736">
+        <v>0.1</v>
+      </c>
+      <c r="G2736">
+        <v>5.37</v>
+      </c>
+      <c r="H2736">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="2737" spans="1:15">
+      <c r="D2737">
+        <v>3</v>
+      </c>
+      <c r="F2737">
+        <v>0.1</v>
+      </c>
+      <c r="G2737">
+        <v>7.44</v>
+      </c>
+      <c r="H2737">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="2738" spans="1:15" s="19" customFormat="1">
+      <c r="E2738" s="36"/>
+    </row>
+    <row r="2739" spans="1:15">
+      <c r="A2739" t="s">
+        <v>392</v>
+      </c>
+      <c r="B2739" s="1">
+        <v>0.57152777777777775</v>
+      </c>
+      <c r="C2739" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2739">
+        <v>1</v>
+      </c>
+      <c r="F2739">
+        <v>0.1</v>
+      </c>
+      <c r="G2739">
+        <v>2.27</v>
+      </c>
+      <c r="H2739">
+        <v>0.04</v>
+      </c>
+      <c r="L2739">
+        <v>13.1</v>
+      </c>
+      <c r="M2739">
+        <v>96.8</v>
+      </c>
+      <c r="N2739">
+        <v>13.21</v>
+      </c>
+      <c r="O2739">
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="2740" spans="1:15">
+      <c r="D2740">
+        <v>2</v>
+      </c>
+      <c r="F2740">
+        <v>0.1</v>
+      </c>
+      <c r="G2740">
+        <v>1.73</v>
+      </c>
+      <c r="H2740">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="2741" spans="1:15">
+      <c r="D2741">
+        <v>3</v>
+      </c>
+      <c r="F2741">
+        <v>0.1</v>
+      </c>
+      <c r="G2741">
+        <v>2.81</v>
+      </c>
+      <c r="H2741">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="2742" spans="1:15">
+      <c r="B2742" s="1">
+        <v>0.55277777777777781</v>
+      </c>
+      <c r="C2742" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2742">
+        <v>1</v>
+      </c>
+      <c r="F2742">
+        <v>0.1</v>
+      </c>
+      <c r="G2742">
+        <v>1.39</v>
+      </c>
+      <c r="H2742">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="L2742">
+        <v>12.9</v>
+      </c>
+      <c r="M2742">
+        <v>95.4</v>
+      </c>
+      <c r="N2742">
+        <v>21.71</v>
+      </c>
+      <c r="O2742">
+        <v>1.48</v>
+      </c>
+    </row>
+    <row r="2743" spans="1:15">
+      <c r="D2743">
+        <v>2</v>
+      </c>
+      <c r="F2743">
+        <v>0.1</v>
+      </c>
+      <c r="G2743">
+        <v>1.04</v>
+      </c>
+      <c r="H2743">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="2744" spans="1:15">
+      <c r="D2744">
+        <v>3</v>
+      </c>
+      <c r="F2744">
+        <v>0.1</v>
+      </c>
+      <c r="G2744">
+        <v>2.27</v>
+      </c>
+      <c r="H2744">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="2745" spans="1:15">
+      <c r="B2745" s="1">
+        <v>0.53541666666666665</v>
+      </c>
+      <c r="C2745" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D2745">
+        <v>1</v>
+      </c>
+      <c r="F2745">
+        <v>19.39</v>
+      </c>
+      <c r="G2745">
+        <v>0</v>
+      </c>
+      <c r="H2745">
+        <v>0</v>
+      </c>
+      <c r="L2745">
+        <v>11.8</v>
+      </c>
+      <c r="M2745">
+        <v>93.9</v>
+      </c>
+      <c r="N2745">
+        <v>13.29</v>
+      </c>
+      <c r="O2745">
+        <v>1.1000000000000001</v>
+      </c>
+    </row>
+    <row r="2746" spans="1:15">
+      <c r="D2746">
+        <v>2</v>
+      </c>
+      <c r="F2746">
+        <v>6.25</v>
+      </c>
+      <c r="G2746">
+        <v>0</v>
+      </c>
+      <c r="H2746">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2747" spans="1:15">
+      <c r="D2747">
+        <v>3</v>
+      </c>
+      <c r="F2747">
+        <v>0.1</v>
+      </c>
+      <c r="G2747">
+        <v>1</v>
+      </c>
+      <c r="H2747">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="2748" spans="1:15">
+      <c r="B2748" s="1">
+        <v>0.52013888888888893</v>
+      </c>
+      <c r="C2748" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D2748">
+        <v>1</v>
+      </c>
+      <c r="F2748">
+        <v>6.25</v>
+      </c>
+      <c r="G2748">
+        <v>3.01</v>
+      </c>
+      <c r="H2748">
+        <v>2.0699999999999998</v>
+      </c>
+      <c r="L2748">
+        <v>12.2</v>
+      </c>
+      <c r="M2748">
+        <v>88.4</v>
+      </c>
+      <c r="N2748">
+        <v>76.72</v>
+      </c>
+      <c r="O2748">
+        <v>9.84</v>
+      </c>
+    </row>
+    <row r="2749" spans="1:15">
+      <c r="D2749">
+        <v>2</v>
+      </c>
+      <c r="F2749">
+        <v>35.82</v>
+      </c>
+      <c r="G2749">
+        <v>1.34</v>
+      </c>
+      <c r="H2749">
+        <v>26.73</v>
+      </c>
+    </row>
+    <row r="2750" spans="1:15">
+      <c r="D2750">
+        <v>3</v>
+      </c>
+      <c r="F2750">
+        <v>96.08</v>
+      </c>
+      <c r="G2750">
+        <v>4.63</v>
+      </c>
+      <c r="H2750">
+        <v>20.75</v>
+      </c>
+    </row>
+    <row r="2751" spans="1:15">
+      <c r="B2751" s="1">
+        <v>0.48888888888888887</v>
+      </c>
+      <c r="C2751" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D2751">
+        <v>1</v>
+      </c>
+      <c r="F2751">
+        <v>0.1</v>
+      </c>
+      <c r="G2751">
+        <v>0.05</v>
+      </c>
+      <c r="H2751">
+        <v>2</v>
+      </c>
+      <c r="L2751">
+        <v>12.6</v>
+      </c>
+      <c r="M2751">
+        <v>96.1</v>
+      </c>
+      <c r="N2751">
+        <v>7.11</v>
+      </c>
+      <c r="O2751">
+        <v>3.56</v>
+      </c>
+    </row>
+    <row r="2752" spans="1:15">
+      <c r="D2752">
+        <v>2</v>
+      </c>
+      <c r="F2752">
+        <v>0.1</v>
+      </c>
+      <c r="G2752">
+        <v>2.77</v>
+      </c>
+      <c r="H2752">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="2753" spans="2:15">
+      <c r="D2753">
+        <v>3</v>
+      </c>
+      <c r="F2753">
+        <v>0.1</v>
+      </c>
+      <c r="G2753">
+        <v>3.95</v>
+      </c>
+      <c r="H2753">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="2754" spans="2:15">
+      <c r="B2754" s="1">
+        <v>0.4826388888888889</v>
+      </c>
+      <c r="C2754" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D2754">
+        <v>1</v>
+      </c>
+      <c r="F2754">
+        <v>0.1</v>
+      </c>
+      <c r="G2754">
+        <v>0.05</v>
+      </c>
+      <c r="H2754">
+        <v>2</v>
+      </c>
+      <c r="L2754">
+        <v>12.2</v>
+      </c>
+      <c r="M2754">
+        <v>99.2</v>
+      </c>
+      <c r="N2754">
+        <v>0.85</v>
+      </c>
+      <c r="O2754">
+        <v>0.26</v>
+      </c>
+    </row>
+    <row r="2755" spans="2:15">
+      <c r="D2755">
+        <v>2</v>
+      </c>
+      <c r="F2755">
+        <v>7.75</v>
+      </c>
+      <c r="G2755">
+        <v>0.6</v>
+      </c>
+      <c r="H2755">
+        <v>12.91</v>
+      </c>
+    </row>
+    <row r="2756" spans="2:15">
+      <c r="D2756">
+        <v>3</v>
+      </c>
+      <c r="F2756">
+        <v>20.170000000000002</v>
+      </c>
+      <c r="G2756">
+        <v>0.75</v>
+      </c>
+      <c r="H2756">
+        <v>26.89</v>
+      </c>
+    </row>
+    <row r="2757" spans="2:15">
+      <c r="B2757" s="1">
+        <v>0.47569444444444442</v>
+      </c>
+      <c r="C2757" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D2757">
+        <v>1</v>
+      </c>
+      <c r="F2757">
+        <v>20.95</v>
+      </c>
+      <c r="G2757">
+        <v>0.8</v>
+      </c>
+      <c r="H2757">
+        <v>26.18</v>
+      </c>
+      <c r="L2757">
+        <v>12.4</v>
+      </c>
+      <c r="M2757">
+        <v>98.6</v>
+      </c>
+      <c r="N2757">
+        <v>0.71</v>
+      </c>
+      <c r="O2757">
+        <v>0.42</v>
+      </c>
+    </row>
+    <row r="2758" spans="2:15">
+      <c r="D2758">
+        <v>2</v>
+      </c>
+      <c r="F2758">
+        <v>79.650000000000006</v>
+      </c>
+      <c r="G2758">
+        <v>1.29</v>
+      </c>
+      <c r="H2758">
+        <v>61.74</v>
+      </c>
+    </row>
+    <row r="2759" spans="2:15">
+      <c r="D2759">
+        <v>3</v>
+      </c>
+      <c r="F2759">
+        <v>25.65</v>
+      </c>
+      <c r="G2759">
+        <v>1.04</v>
+      </c>
+      <c r="H2759">
+        <v>24.66</v>
+      </c>
+    </row>
+    <row r="2760" spans="2:15">
+      <c r="B2760" s="1">
+        <v>0.41041666666666665</v>
+      </c>
+      <c r="C2760" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D2760">
+        <v>1</v>
+      </c>
+      <c r="F2760">
+        <v>34.25</v>
+      </c>
+      <c r="G2760">
+        <v>0.95</v>
+      </c>
+      <c r="H2760">
+        <v>36.06</v>
+      </c>
+      <c r="L2760">
+        <v>11</v>
+      </c>
+      <c r="M2760">
+        <v>97.3</v>
+      </c>
+      <c r="N2760">
+        <v>0.92</v>
+      </c>
+      <c r="O2760">
+        <v>0.21</v>
+      </c>
+    </row>
+    <row r="2761" spans="2:15">
+      <c r="D2761">
+        <v>2</v>
+      </c>
+      <c r="F2761">
+        <v>7.75</v>
+      </c>
+      <c r="G2761">
+        <v>0.4</v>
+      </c>
+      <c r="H2761">
+        <v>19.37</v>
+      </c>
+    </row>
+    <row r="2762" spans="2:15">
+      <c r="D2762">
+        <v>3</v>
+      </c>
+      <c r="F2762">
+        <v>40.520000000000003</v>
+      </c>
+      <c r="G2762">
+        <v>1.29</v>
+      </c>
+      <c r="H2762">
+        <v>31.41</v>
+      </c>
+    </row>
+    <row r="2763" spans="2:15">
+      <c r="B2763" s="1">
+        <v>0.4548611111111111</v>
+      </c>
+      <c r="C2763" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="D2763">
+        <v>1</v>
+      </c>
+      <c r="F2763">
+        <v>0.1</v>
+      </c>
+      <c r="G2763">
+        <v>0.3</v>
+      </c>
+      <c r="H2763">
+        <v>0.33</v>
+      </c>
+      <c r="L2763">
+        <v>12.2</v>
+      </c>
+      <c r="M2763">
+        <v>98.7</v>
+      </c>
+      <c r="N2763">
+        <v>0.81</v>
+      </c>
+      <c r="O2763">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="2764" spans="2:15">
+      <c r="D2764">
+        <v>2</v>
+      </c>
+      <c r="F2764">
+        <v>36.6</v>
+      </c>
+      <c r="G2764">
+        <v>0.75</v>
+      </c>
+      <c r="H2764">
+        <v>48.8</v>
+      </c>
+    </row>
+    <row r="2765" spans="2:15">
+      <c r="D2765">
+        <v>3</v>
+      </c>
+      <c r="F2765">
+        <v>39.729999999999997</v>
+      </c>
+      <c r="G2765">
+        <v>0.85</v>
+      </c>
+      <c r="H2765">
+        <v>46.74</v>
+      </c>
+    </row>
+    <row r="2766" spans="2:15">
+      <c r="B2766" s="1">
+        <v>0.58888888888888891</v>
+      </c>
+      <c r="C2766" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="D2766">
+        <v>1</v>
+      </c>
+      <c r="F2766">
+        <v>0.1</v>
+      </c>
+      <c r="G2766">
+        <v>1.63</v>
+      </c>
+      <c r="H2766">
+        <v>0.06</v>
+      </c>
+      <c r="L2766">
+        <v>15.3</v>
+      </c>
+      <c r="M2766">
+        <v>97.6</v>
+      </c>
+      <c r="N2766">
+        <v>0.84</v>
+      </c>
+      <c r="O2766">
+        <v>0.66</v>
+      </c>
+    </row>
+    <row r="2767" spans="2:15">
+      <c r="C2767" s="3"/>
+      <c r="D2767">
+        <v>2</v>
+      </c>
+      <c r="F2767">
+        <v>0.1</v>
+      </c>
+      <c r="G2767">
+        <v>1.0900000000000001</v>
+      </c>
+      <c r="H2767">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="2768" spans="2:15">
+      <c r="D2768">
+        <v>3</v>
+      </c>
+      <c r="F2768">
+        <v>0.1</v>
+      </c>
+      <c r="G2768">
+        <v>1.73</v>
+      </c>
+      <c r="H2768">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="2769" spans="5:5" s="19" customFormat="1">
+      <c r="E2769" s="36"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Daily TALT data update 2025-09-04
</commit_message>
<xml_diff>
--- a/data/talt_cyano/talt_cyano_digitized.xlsx
+++ b/data/talt_cyano/talt_cyano_digitized.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29212"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29225"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="20435" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ED0097AE-E8BF-4194-85E9-A632FE632A20}"/>
+  <xr:revisionPtr revIDLastSave="20831" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CE9692C1-B11D-466F-9214-9CC4539DAEFC}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1854" uniqueCount="390">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1878" uniqueCount="393">
   <si>
     <t>Date</t>
   </si>
@@ -1197,10 +1197,19 @@
     <t xml:space="preserve">18/08/2025 </t>
   </si>
   <si>
+    <t xml:space="preserve">0.34	</t>
+  </si>
+  <si>
     <t xml:space="preserve">20/08/2025 </t>
   </si>
   <si>
     <t xml:space="preserve">22/08/2025 </t>
+  </si>
+  <si>
+    <t>25/08/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">29/08/2025 </t>
   </si>
 </sst>
 </file>
@@ -1758,7 +1767,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S2707"/>
+  <dimension ref="A1:S2769"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="11.7109375" customWidth="1"/>
@@ -68701,6 +68710,9 @@
       <c r="A2615" t="s">
         <v>387</v>
       </c>
+      <c r="B2615" s="1">
+        <v>0.43541666666666667</v>
+      </c>
       <c r="C2615" s="3" t="s">
         <v>20</v>
       </c>
@@ -68719,6 +68731,18 @@
       <c r="H2615">
         <v>0</v>
       </c>
+      <c r="L2615">
+        <v>11.3</v>
+      </c>
+      <c r="M2615">
+        <v>98.4</v>
+      </c>
+      <c r="N2615">
+        <v>1.01</v>
+      </c>
+      <c r="O2615" t="s">
+        <v>388</v>
+      </c>
       <c r="P2615" t="s">
         <v>319</v>
       </c>
@@ -68752,6 +68776,9 @@
       </c>
     </row>
     <row r="2618" spans="1:18">
+      <c r="B2618" s="1">
+        <v>0.45694444444444443</v>
+      </c>
       <c r="C2618" s="3" t="s">
         <v>25</v>
       </c>
@@ -68767,6 +68794,18 @@
       <c r="H2618">
         <v>0</v>
       </c>
+      <c r="L2618">
+        <v>12.6</v>
+      </c>
+      <c r="M2618">
+        <v>88.4</v>
+      </c>
+      <c r="N2618">
+        <v>2.84</v>
+      </c>
+      <c r="O2618">
+        <v>0.17</v>
+      </c>
     </row>
     <row r="2619" spans="1:18">
       <c r="D2619">
@@ -68797,6 +68836,9 @@
       </c>
     </row>
     <row r="2621" spans="1:18">
+      <c r="B2621" s="1">
+        <v>0.47430555555555554</v>
+      </c>
       <c r="C2621" s="3" t="s">
         <v>27</v>
       </c>
@@ -68812,6 +68854,18 @@
       <c r="H2621">
         <v>0.09</v>
       </c>
+      <c r="L2621">
+        <v>11.3</v>
+      </c>
+      <c r="M2621">
+        <v>99</v>
+      </c>
+      <c r="N2621">
+        <v>2.12</v>
+      </c>
+      <c r="O2621">
+        <v>0.22</v>
+      </c>
     </row>
     <row r="2622" spans="1:18">
       <c r="D2622">
@@ -68842,6 +68896,9 @@
       </c>
     </row>
     <row r="2624" spans="1:18">
+      <c r="B2624" s="1">
+        <v>0.49236111111111114</v>
+      </c>
       <c r="C2624" s="3" t="s">
         <v>58</v>
       </c>
@@ -68857,8 +68914,20 @@
       <c r="H2624">
         <v>2</v>
       </c>
-    </row>
-    <row r="2625" spans="3:8">
+      <c r="L2624">
+        <v>11.7</v>
+      </c>
+      <c r="M2624">
+        <v>90.6</v>
+      </c>
+      <c r="N2624">
+        <v>7.08</v>
+      </c>
+      <c r="O2624">
+        <v>4.43</v>
+      </c>
+    </row>
+    <row r="2625" spans="2:15">
       <c r="D2625">
         <v>2</v>
       </c>
@@ -68872,7 +68941,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2626" spans="3:8">
+    <row r="2626" spans="2:15">
       <c r="D2626">
         <v>3</v>
       </c>
@@ -68886,7 +68955,10 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="2627" spans="3:8">
+    <row r="2627" spans="2:15">
+      <c r="B2627" s="1">
+        <v>0.50694444444444442</v>
+      </c>
       <c r="C2627" s="3" t="s">
         <v>29</v>
       </c>
@@ -68902,8 +68974,20 @@
       <c r="H2627">
         <v>0</v>
       </c>
-    </row>
-    <row r="2628" spans="3:8">
+      <c r="L2627">
+        <v>11.8</v>
+      </c>
+      <c r="M2627">
+        <v>111.2</v>
+      </c>
+      <c r="N2627">
+        <v>0.86</v>
+      </c>
+      <c r="O2627">
+        <v>0.17</v>
+      </c>
+    </row>
+    <row r="2628" spans="2:15">
       <c r="D2628">
         <v>2</v>
       </c>
@@ -68917,7 +69001,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2629" spans="3:8">
+    <row r="2629" spans="2:15">
       <c r="D2629">
         <v>3</v>
       </c>
@@ -68931,7 +69015,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2630" spans="3:8">
+    <row r="2630" spans="2:15">
+      <c r="B2630" s="1">
+        <v>0.51597222222222228</v>
+      </c>
       <c r="C2630" s="3" t="s">
         <v>30</v>
       </c>
@@ -68947,8 +69034,20 @@
       <c r="H2630">
         <v>0</v>
       </c>
-    </row>
-    <row r="2631" spans="3:8">
+      <c r="L2630">
+        <v>11.9</v>
+      </c>
+      <c r="M2630">
+        <v>105</v>
+      </c>
+      <c r="N2630">
+        <v>0.54</v>
+      </c>
+      <c r="O2630">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="2631" spans="2:15">
       <c r="D2631">
         <v>2</v>
       </c>
@@ -68962,7 +69061,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2632" spans="3:8">
+    <row r="2632" spans="2:15">
       <c r="D2632">
         <v>3</v>
       </c>
@@ -68976,7 +69075,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2633" spans="3:8">
+    <row r="2633" spans="2:15">
+      <c r="B2633" s="1">
+        <v>0.52916666666666667</v>
+      </c>
       <c r="C2633" s="3" t="s">
         <v>31</v>
       </c>
@@ -68992,8 +69094,20 @@
       <c r="H2633">
         <v>0</v>
       </c>
-    </row>
-    <row r="2634" spans="3:8">
+      <c r="L2633">
+        <v>12.3</v>
+      </c>
+      <c r="M2633">
+        <v>102.9</v>
+      </c>
+      <c r="N2633">
+        <v>0.31</v>
+      </c>
+      <c r="O2633">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="2634" spans="2:15">
       <c r="D2634">
         <v>2</v>
       </c>
@@ -69007,7 +69121,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2635" spans="3:8">
+    <row r="2635" spans="2:15">
       <c r="D2635">
         <v>3</v>
       </c>
@@ -69021,7 +69135,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2636" spans="3:8">
+    <row r="2636" spans="2:15">
+      <c r="B2636" s="1">
+        <v>0.54305555555555551</v>
+      </c>
       <c r="C2636" s="3" t="s">
         <v>32</v>
       </c>
@@ -69037,8 +69154,20 @@
       <c r="H2636">
         <v>0.03</v>
       </c>
-    </row>
-    <row r="2637" spans="3:8">
+      <c r="L2636">
+        <v>11.9</v>
+      </c>
+      <c r="M2636">
+        <v>100.4</v>
+      </c>
+      <c r="N2636">
+        <v>0.87</v>
+      </c>
+      <c r="O2636">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="2637" spans="2:15">
       <c r="D2637">
         <v>2</v>
       </c>
@@ -69052,7 +69181,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2638" spans="3:8">
+    <row r="2638" spans="2:15">
       <c r="D2638">
         <v>3</v>
       </c>
@@ -69066,7 +69195,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2639" spans="3:8">
+    <row r="2639" spans="2:15">
+      <c r="B2639" s="1">
+        <v>0.56666666666666665</v>
+      </c>
       <c r="C2639" s="3" t="s">
         <v>41</v>
       </c>
@@ -69082,8 +69214,20 @@
       <c r="H2639">
         <v>0</v>
       </c>
-    </row>
-    <row r="2640" spans="3:8">
+      <c r="L2639">
+        <v>12.5</v>
+      </c>
+      <c r="M2639">
+        <v>103.4</v>
+      </c>
+      <c r="N2639">
+        <v>1.34</v>
+      </c>
+      <c r="O2639">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="2640" spans="2:15">
       <c r="D2640">
         <v>2</v>
       </c>
@@ -69112,6 +69256,9 @@
       </c>
     </row>
     <row r="2642" spans="1:16">
+      <c r="B2642" s="1">
+        <v>0.5756944444444444</v>
+      </c>
       <c r="C2642" s="3" t="s">
         <v>34</v>
       </c>
@@ -69126,6 +69273,18 @@
       </c>
       <c r="H2642">
         <v>0</v>
+      </c>
+      <c r="L2642">
+        <v>13.2</v>
+      </c>
+      <c r="M2642">
+        <v>94.1</v>
+      </c>
+      <c r="N2642">
+        <v>2.4700000000000002</v>
+      </c>
+      <c r="O2642">
+        <v>0.27</v>
       </c>
     </row>
     <row r="2643" spans="1:16">
@@ -69162,7 +69321,10 @@
     </row>
     <row r="2646" spans="1:16">
       <c r="A2646" t="s">
-        <v>388</v>
+        <v>389</v>
+      </c>
+      <c r="B2646" s="1">
+        <v>0.48958333333333331</v>
       </c>
       <c r="C2646" s="3" t="s">
         <v>20</v>
@@ -69182,6 +69344,18 @@
       <c r="H2646">
         <v>0</v>
       </c>
+      <c r="L2646">
+        <v>10.8</v>
+      </c>
+      <c r="M2646">
+        <v>90.6</v>
+      </c>
+      <c r="N2646">
+        <v>4.1500000000000004</v>
+      </c>
+      <c r="O2646">
+        <v>0.08</v>
+      </c>
       <c r="P2646" t="s">
         <v>147</v>
       </c>
@@ -69215,6 +69389,9 @@
       </c>
     </row>
     <row r="2649" spans="1:16">
+      <c r="B2649" s="1">
+        <v>0.50069444444444444</v>
+      </c>
       <c r="C2649" s="3" t="s">
         <v>25</v>
       </c>
@@ -69230,6 +69407,18 @@
       <c r="H2649">
         <v>0</v>
       </c>
+      <c r="L2649">
+        <v>10.8</v>
+      </c>
+      <c r="M2649">
+        <v>95.8</v>
+      </c>
+      <c r="N2649">
+        <v>4.93</v>
+      </c>
+      <c r="O2649">
+        <v>0.15</v>
+      </c>
     </row>
     <row r="2650" spans="1:16">
       <c r="D2650">
@@ -69260,6 +69449,9 @@
       </c>
     </row>
     <row r="2652" spans="1:16">
+      <c r="B2652" s="1">
+        <v>0.51597222222222228</v>
+      </c>
       <c r="C2652" s="3" t="s">
         <v>27</v>
       </c>
@@ -69275,6 +69467,18 @@
       <c r="H2652">
         <v>0</v>
       </c>
+      <c r="L2652">
+        <v>9.9</v>
+      </c>
+      <c r="M2652">
+        <v>97.1</v>
+      </c>
+      <c r="N2652">
+        <v>10.51</v>
+      </c>
+      <c r="O2652">
+        <v>0.28000000000000003</v>
+      </c>
     </row>
     <row r="2653" spans="1:16">
       <c r="D2653">
@@ -69305,6 +69509,9 @@
       </c>
     </row>
     <row r="2655" spans="1:16">
+      <c r="B2655" s="1">
+        <v>0.52569444444444446</v>
+      </c>
       <c r="C2655" s="3" t="s">
         <v>58</v>
       </c>
@@ -69320,6 +69527,18 @@
       <c r="H2655">
         <v>0.15</v>
       </c>
+      <c r="L2655">
+        <v>9.3000000000000007</v>
+      </c>
+      <c r="M2655">
+        <v>99.3</v>
+      </c>
+      <c r="N2655">
+        <v>13.22</v>
+      </c>
+      <c r="O2655">
+        <v>0.91</v>
+      </c>
     </row>
     <row r="2656" spans="1:16">
       <c r="D2656">
@@ -69335,7 +69554,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2657" spans="3:8">
+    <row r="2657" spans="2:15">
       <c r="D2657">
         <v>3</v>
       </c>
@@ -69349,7 +69568,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2658" spans="3:8">
+    <row r="2658" spans="2:15">
+      <c r="B2658" s="1">
+        <v>0.53611111111111109</v>
+      </c>
       <c r="C2658" s="3" t="s">
         <v>29</v>
       </c>
@@ -69365,8 +69587,20 @@
       <c r="H2658">
         <v>7.0000000000000007E-2</v>
       </c>
-    </row>
-    <row r="2659" spans="3:8">
+      <c r="L2658">
+        <v>9.3000000000000007</v>
+      </c>
+      <c r="M2658">
+        <v>101.3</v>
+      </c>
+      <c r="N2658">
+        <v>15.49</v>
+      </c>
+      <c r="O2658">
+        <v>2.31</v>
+      </c>
+    </row>
+    <row r="2659" spans="2:15">
       <c r="D2659">
         <v>2</v>
       </c>
@@ -69380,7 +69614,7 @@
         <v>0.08</v>
       </c>
     </row>
-    <row r="2660" spans="3:8">
+    <row r="2660" spans="2:15">
       <c r="D2660">
         <v>3</v>
       </c>
@@ -69394,7 +69628,10 @@
         <v>0.08</v>
       </c>
     </row>
-    <row r="2661" spans="3:8">
+    <row r="2661" spans="2:15">
+      <c r="B2661" s="1">
+        <v>0.54652777777777772</v>
+      </c>
       <c r="C2661" s="3" t="s">
         <v>30</v>
       </c>
@@ -69410,8 +69647,20 @@
       <c r="H2661">
         <v>18.75</v>
       </c>
-    </row>
-    <row r="2662" spans="3:8">
+      <c r="L2661">
+        <v>9.3000000000000007</v>
+      </c>
+      <c r="M2661">
+        <v>96.7</v>
+      </c>
+      <c r="N2661">
+        <v>20.260000000000002</v>
+      </c>
+      <c r="O2661">
+        <v>3.07</v>
+      </c>
+    </row>
+    <row r="2662" spans="2:15">
       <c r="D2662">
         <v>2</v>
       </c>
@@ -69425,7 +69674,7 @@
         <v>9.0500000000000007</v>
       </c>
     </row>
-    <row r="2663" spans="3:8">
+    <row r="2663" spans="2:15">
       <c r="D2663">
         <v>3</v>
       </c>
@@ -69439,7 +69688,10 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="2664" spans="3:8">
+    <row r="2664" spans="2:15">
+      <c r="B2664" s="1">
+        <v>0.5541666666666667</v>
+      </c>
       <c r="C2664" s="3" t="s">
         <v>31</v>
       </c>
@@ -69455,8 +69707,20 @@
       <c r="H2664">
         <v>0</v>
       </c>
-    </row>
-    <row r="2665" spans="3:8">
+      <c r="L2664">
+        <v>12.6</v>
+      </c>
+      <c r="M2664">
+        <v>102.8</v>
+      </c>
+      <c r="N2664">
+        <v>3.31</v>
+      </c>
+      <c r="O2664">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="2665" spans="2:15">
       <c r="D2665">
         <v>2</v>
       </c>
@@ -69470,7 +69734,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2666" spans="3:8">
+    <row r="2666" spans="2:15">
       <c r="D2666">
         <v>3</v>
       </c>
@@ -69484,7 +69748,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2667" spans="3:8">
+    <row r="2667" spans="2:15">
+      <c r="B2667" s="1">
+        <v>0.56111111111111112</v>
+      </c>
       <c r="C2667" s="3" t="s">
         <v>32</v>
       </c>
@@ -69500,8 +69767,20 @@
       <c r="H2667">
         <v>0</v>
       </c>
-    </row>
-    <row r="2668" spans="3:8">
+      <c r="L2667">
+        <v>10.4</v>
+      </c>
+      <c r="M2667">
+        <v>98.8</v>
+      </c>
+      <c r="N2667">
+        <v>9.1199999999999992</v>
+      </c>
+      <c r="O2667">
+        <v>0.32</v>
+      </c>
+    </row>
+    <row r="2668" spans="2:15">
       <c r="D2668">
         <v>2</v>
       </c>
@@ -69515,7 +69794,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2669" spans="3:8">
+    <row r="2669" spans="2:15">
       <c r="D2669">
         <v>3</v>
       </c>
@@ -69529,7 +69808,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2670" spans="3:8">
+    <row r="2670" spans="2:15">
+      <c r="B2670" s="1">
+        <v>0.57708333333333328</v>
+      </c>
       <c r="C2670" s="3" t="s">
         <v>41</v>
       </c>
@@ -69545,8 +69827,20 @@
       <c r="H2670">
         <v>0</v>
       </c>
-    </row>
-    <row r="2671" spans="3:8">
+      <c r="L2670">
+        <v>11.5</v>
+      </c>
+      <c r="M2670">
+        <v>105.1</v>
+      </c>
+      <c r="N2670">
+        <v>1.66</v>
+      </c>
+      <c r="O2670">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="2671" spans="2:15">
       <c r="D2671">
         <v>2</v>
       </c>
@@ -69560,7 +69854,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2672" spans="3:8">
+    <row r="2672" spans="2:15">
       <c r="D2672">
         <v>3</v>
       </c>
@@ -69575,6 +69869,9 @@
       </c>
     </row>
     <row r="2673" spans="1:16">
+      <c r="B2673" s="1">
+        <v>0.58333333333333337</v>
+      </c>
       <c r="C2673" s="3" t="s">
         <v>34</v>
       </c>
@@ -69589,6 +69886,18 @@
       </c>
       <c r="H2673">
         <v>0</v>
+      </c>
+      <c r="L2673">
+        <v>11</v>
+      </c>
+      <c r="M2673">
+        <v>96.6</v>
+      </c>
+      <c r="N2673">
+        <v>1.94</v>
+      </c>
+      <c r="O2673">
+        <v>0.04</v>
       </c>
     </row>
     <row r="2674" spans="1:16">
@@ -69625,7 +69934,10 @@
     </row>
     <row r="2677" spans="1:16">
       <c r="A2677" t="s">
-        <v>389</v>
+        <v>390</v>
+      </c>
+      <c r="B2677" s="1">
+        <v>0.50069444444444444</v>
       </c>
       <c r="C2677" s="3" t="s">
         <v>20</v>
@@ -69645,6 +69957,18 @@
       <c r="H2677">
         <v>0</v>
       </c>
+      <c r="L2677">
+        <v>12.2</v>
+      </c>
+      <c r="M2677">
+        <v>95.7</v>
+      </c>
+      <c r="N2677">
+        <v>1.1399999999999999</v>
+      </c>
+      <c r="O2677">
+        <v>0.08</v>
+      </c>
       <c r="P2677" t="s">
         <v>157</v>
       </c>
@@ -69678,6 +70002,9 @@
       </c>
     </row>
     <row r="2680" spans="1:16">
+      <c r="B2680" s="1">
+        <v>0.5180555555555556</v>
+      </c>
       <c r="C2680" s="3" t="s">
         <v>25</v>
       </c>
@@ -69693,6 +70020,18 @@
       <c r="H2680">
         <v>0</v>
       </c>
+      <c r="L2680">
+        <v>11.3</v>
+      </c>
+      <c r="M2680">
+        <v>100.3</v>
+      </c>
+      <c r="N2680">
+        <v>1.94</v>
+      </c>
+      <c r="O2680">
+        <v>0.15</v>
+      </c>
     </row>
     <row r="2681" spans="1:16">
       <c r="D2681">
@@ -69723,6 +70062,9 @@
       </c>
     </row>
     <row r="2683" spans="1:16">
+      <c r="B2683" s="1">
+        <v>0.57152777777777775</v>
+      </c>
       <c r="C2683" s="3" t="s">
         <v>27</v>
       </c>
@@ -69738,6 +70080,18 @@
       <c r="H2683">
         <v>0</v>
       </c>
+      <c r="L2683">
+        <v>11.5</v>
+      </c>
+      <c r="M2683">
+        <v>92.8</v>
+      </c>
+      <c r="N2683">
+        <v>1.75</v>
+      </c>
+      <c r="O2683">
+        <v>0.06</v>
+      </c>
     </row>
     <row r="2684" spans="1:16">
       <c r="D2684">
@@ -69768,6 +70122,9 @@
       </c>
     </row>
     <row r="2686" spans="1:16">
+      <c r="B2686" s="1">
+        <v>0.58958333333333335</v>
+      </c>
       <c r="C2686" s="3" t="s">
         <v>58</v>
       </c>
@@ -69783,6 +70140,18 @@
       <c r="H2686">
         <v>0</v>
       </c>
+      <c r="L2686">
+        <v>10.9</v>
+      </c>
+      <c r="M2686">
+        <v>102.5</v>
+      </c>
+      <c r="N2686">
+        <v>1.41</v>
+      </c>
+      <c r="O2686">
+        <v>0.05</v>
+      </c>
     </row>
     <row r="2687" spans="1:16">
       <c r="D2687">
@@ -69812,7 +70181,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2689" spans="3:8">
+    <row r="2689" spans="2:15">
+      <c r="B2689" s="1">
+        <v>0.61319444444444449</v>
+      </c>
       <c r="C2689" s="3" t="s">
         <v>29</v>
       </c>
@@ -69828,8 +70200,20 @@
       <c r="H2689">
         <v>0</v>
       </c>
-    </row>
-    <row r="2690" spans="3:8">
+      <c r="L2689">
+        <v>10.7</v>
+      </c>
+      <c r="M2689">
+        <v>103.6</v>
+      </c>
+      <c r="N2689">
+        <v>4.34</v>
+      </c>
+      <c r="O2689">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="2690" spans="2:15">
       <c r="D2690">
         <v>2</v>
       </c>
@@ -69843,7 +70227,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2691" spans="3:8">
+    <row r="2691" spans="2:15">
       <c r="D2691">
         <v>3</v>
       </c>
@@ -69857,7 +70241,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2692" spans="3:8">
+    <row r="2692" spans="2:15">
+      <c r="B2692" s="1">
+        <v>0.63194444444444442</v>
+      </c>
       <c r="C2692" s="3" t="s">
         <v>30</v>
       </c>
@@ -69873,8 +70260,20 @@
       <c r="H2692">
         <v>0.28000000000000003</v>
       </c>
-    </row>
-    <row r="2693" spans="3:8">
+      <c r="L2692">
+        <v>11</v>
+      </c>
+      <c r="M2692">
+        <v>104.3</v>
+      </c>
+      <c r="N2692">
+        <v>2.39</v>
+      </c>
+      <c r="O2692">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="2693" spans="2:15">
       <c r="D2693">
         <v>2</v>
       </c>
@@ -69888,7 +70287,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2694" spans="3:8">
+    <row r="2694" spans="2:15">
       <c r="D2694">
         <v>3</v>
       </c>
@@ -69902,7 +70301,10 @@
         <v>13.18</v>
       </c>
     </row>
-    <row r="2695" spans="3:8">
+    <row r="2695" spans="2:15">
+      <c r="B2695" s="1">
+        <v>0.64513888888888893</v>
+      </c>
       <c r="C2695" s="3" t="s">
         <v>31</v>
       </c>
@@ -69918,8 +70320,20 @@
       <c r="H2695">
         <v>0</v>
       </c>
-    </row>
-    <row r="2696" spans="3:8">
+      <c r="L2695">
+        <v>12</v>
+      </c>
+      <c r="M2695">
+        <v>101.6</v>
+      </c>
+      <c r="N2695">
+        <v>1.49</v>
+      </c>
+      <c r="O2695">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="2696" spans="2:15">
       <c r="D2696">
         <v>2</v>
       </c>
@@ -69933,7 +70347,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2697" spans="3:8">
+    <row r="2697" spans="2:15">
       <c r="D2697">
         <v>3</v>
       </c>
@@ -69947,7 +70361,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2698" spans="3:8">
+    <row r="2698" spans="2:15">
+      <c r="B2698" s="1">
+        <v>0.65833333333333333</v>
+      </c>
       <c r="C2698" s="3" t="s">
         <v>32</v>
       </c>
@@ -69963,8 +70380,20 @@
       <c r="H2698">
         <v>0</v>
       </c>
-    </row>
-    <row r="2699" spans="3:8">
+      <c r="L2698">
+        <v>11.6</v>
+      </c>
+      <c r="M2698">
+        <v>105.6</v>
+      </c>
+      <c r="N2698">
+        <v>1.98</v>
+      </c>
+      <c r="O2698">
+        <v>0.19</v>
+      </c>
+    </row>
+    <row r="2699" spans="2:15">
       <c r="D2699">
         <v>2</v>
       </c>
@@ -69978,7 +70407,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2700" spans="3:8">
+    <row r="2700" spans="2:15">
       <c r="D2700">
         <v>3</v>
       </c>
@@ -69992,7 +70421,10 @@
         <v>0.28000000000000003</v>
       </c>
     </row>
-    <row r="2701" spans="3:8">
+    <row r="2701" spans="2:15">
+      <c r="B2701" s="1">
+        <v>0.67222222222222228</v>
+      </c>
       <c r="C2701" s="3" t="s">
         <v>41</v>
       </c>
@@ -70008,8 +70440,20 @@
       <c r="H2701">
         <v>0.04</v>
       </c>
-    </row>
-    <row r="2702" spans="3:8">
+      <c r="L2701">
+        <v>12.6</v>
+      </c>
+      <c r="M2701">
+        <v>105.8</v>
+      </c>
+      <c r="N2701">
+        <v>6.63</v>
+      </c>
+      <c r="O2701">
+        <v>0.92</v>
+      </c>
+    </row>
+    <row r="2702" spans="2:15">
       <c r="D2702">
         <v>2</v>
       </c>
@@ -70023,7 +70467,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="2703" spans="3:8">
+    <row r="2703" spans="2:15">
       <c r="D2703">
         <v>3</v>
       </c>
@@ -70037,7 +70481,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="2704" spans="3:8">
+    <row r="2704" spans="2:15">
       <c r="C2704" s="3" t="s">
         <v>34</v>
       </c>
@@ -70053,8 +70497,20 @@
       <c r="H2704">
         <v>0</v>
       </c>
-    </row>
-    <row r="2705" spans="3:8">
+      <c r="L2704">
+        <v>14.3</v>
+      </c>
+      <c r="M2704">
+        <v>106.6</v>
+      </c>
+      <c r="N2704">
+        <v>9.81</v>
+      </c>
+      <c r="O2704">
+        <v>0.82</v>
+      </c>
+    </row>
+    <row r="2705" spans="1:15">
       <c r="C2705" s="3"/>
       <c r="D2705">
         <v>2</v>
@@ -70069,7 +70525,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2706" spans="3:8">
+    <row r="2706" spans="1:15">
       <c r="D2706">
         <v>3</v>
       </c>
@@ -70083,8 +70539,1225 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2707" spans="3:8" s="19" customFormat="1">
+    <row r="2707" spans="1:15" s="19" customFormat="1">
       <c r="E2707" s="36"/>
+    </row>
+    <row r="2708" spans="1:15">
+      <c r="A2708" t="s">
+        <v>391</v>
+      </c>
+      <c r="B2708" s="1">
+        <v>0.55833333333333335</v>
+      </c>
+      <c r="C2708" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2708">
+        <v>1</v>
+      </c>
+      <c r="E2708" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F2708">
+        <v>0.1</v>
+      </c>
+      <c r="G2708">
+        <v>0</v>
+      </c>
+      <c r="H2708">
+        <v>0</v>
+      </c>
+      <c r="L2708">
+        <v>12.5</v>
+      </c>
+      <c r="M2708">
+        <v>97.5</v>
+      </c>
+      <c r="N2708">
+        <v>0.98</v>
+      </c>
+      <c r="O2708">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="2709" spans="1:15">
+      <c r="D2709">
+        <v>2</v>
+      </c>
+      <c r="F2709">
+        <v>0.1</v>
+      </c>
+      <c r="G2709">
+        <v>0</v>
+      </c>
+      <c r="H2709">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2710" spans="1:15">
+      <c r="D2710">
+        <v>3</v>
+      </c>
+      <c r="F2710">
+        <v>0.1</v>
+      </c>
+      <c r="G2710">
+        <v>0</v>
+      </c>
+      <c r="H2710">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2711" spans="1:15">
+      <c r="B2711" s="1">
+        <v>0.57013888888888886</v>
+      </c>
+      <c r="C2711" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2711">
+        <v>1</v>
+      </c>
+      <c r="F2711">
+        <v>0.1</v>
+      </c>
+      <c r="G2711">
+        <v>0</v>
+      </c>
+      <c r="H2711">
+        <v>0</v>
+      </c>
+      <c r="L2711">
+        <v>11.7</v>
+      </c>
+      <c r="M2711">
+        <v>95.2</v>
+      </c>
+      <c r="N2711">
+        <v>3.69</v>
+      </c>
+      <c r="O2711">
+        <v>0.14000000000000001</v>
+      </c>
+    </row>
+    <row r="2712" spans="1:15">
+      <c r="D2712">
+        <v>2</v>
+      </c>
+      <c r="F2712">
+        <v>0.1</v>
+      </c>
+      <c r="G2712">
+        <v>0</v>
+      </c>
+      <c r="H2712">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2713" spans="1:15">
+      <c r="D2713">
+        <v>3</v>
+      </c>
+      <c r="F2713">
+        <v>0.1</v>
+      </c>
+      <c r="G2713">
+        <v>0</v>
+      </c>
+      <c r="H2713">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2714" spans="1:15">
+      <c r="B2714" s="1">
+        <v>0.57986111111111116</v>
+      </c>
+      <c r="C2714" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D2714">
+        <v>1</v>
+      </c>
+      <c r="F2714">
+        <v>0.1</v>
+      </c>
+      <c r="G2714">
+        <v>0</v>
+      </c>
+      <c r="H2714">
+        <v>0</v>
+      </c>
+      <c r="L2714">
+        <v>11.1</v>
+      </c>
+      <c r="M2714">
+        <v>100.1</v>
+      </c>
+      <c r="N2714">
+        <v>0.76</v>
+      </c>
+      <c r="O2714">
+        <v>0.44</v>
+      </c>
+    </row>
+    <row r="2715" spans="1:15">
+      <c r="D2715">
+        <v>2</v>
+      </c>
+      <c r="F2715">
+        <v>0.1</v>
+      </c>
+      <c r="G2715">
+        <v>0</v>
+      </c>
+      <c r="H2715">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2716" spans="1:15">
+      <c r="D2716">
+        <v>3</v>
+      </c>
+      <c r="F2716">
+        <v>0.1</v>
+      </c>
+      <c r="G2716">
+        <v>0</v>
+      </c>
+      <c r="H2716">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2717" spans="1:15">
+      <c r="B2717" s="1">
+        <v>0.59097222222222223</v>
+      </c>
+      <c r="C2717" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D2717">
+        <v>1</v>
+      </c>
+      <c r="F2717">
+        <v>0.1</v>
+      </c>
+      <c r="G2717">
+        <v>0</v>
+      </c>
+      <c r="H2717">
+        <v>0</v>
+      </c>
+      <c r="L2717">
+        <v>11.5</v>
+      </c>
+      <c r="M2717">
+        <v>101.3</v>
+      </c>
+      <c r="N2717">
+        <v>0.64</v>
+      </c>
+      <c r="O2717">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="2718" spans="1:15">
+      <c r="D2718">
+        <v>2</v>
+      </c>
+      <c r="F2718">
+        <v>0.1</v>
+      </c>
+      <c r="G2718">
+        <v>0</v>
+      </c>
+      <c r="H2718">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2719" spans="1:15">
+      <c r="D2719">
+        <v>3</v>
+      </c>
+      <c r="F2719">
+        <v>0.1</v>
+      </c>
+      <c r="G2719">
+        <v>0</v>
+      </c>
+      <c r="H2719">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2720" spans="1:15">
+      <c r="B2720" s="1">
+        <v>0.60277777777777775</v>
+      </c>
+      <c r="C2720" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D2720">
+        <v>1</v>
+      </c>
+      <c r="F2720">
+        <v>0.1</v>
+      </c>
+      <c r="G2720">
+        <v>0</v>
+      </c>
+      <c r="H2720">
+        <v>0</v>
+      </c>
+      <c r="L2720">
+        <v>11.4</v>
+      </c>
+      <c r="M2720">
+        <v>108.2</v>
+      </c>
+      <c r="N2720">
+        <v>0.68</v>
+      </c>
+      <c r="O2720">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="2721" spans="2:15">
+      <c r="D2721">
+        <v>2</v>
+      </c>
+      <c r="F2721">
+        <v>0.1</v>
+      </c>
+      <c r="G2721">
+        <v>0</v>
+      </c>
+      <c r="H2721">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2722" spans="2:15">
+      <c r="D2722">
+        <v>3</v>
+      </c>
+      <c r="F2722">
+        <v>0.1</v>
+      </c>
+      <c r="G2722">
+        <v>0</v>
+      </c>
+      <c r="H2722">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2723" spans="2:15">
+      <c r="B2723" s="1">
+        <v>0.60833333333333328</v>
+      </c>
+      <c r="C2723" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D2723">
+        <v>1</v>
+      </c>
+      <c r="F2723">
+        <v>0.1</v>
+      </c>
+      <c r="G2723">
+        <v>0</v>
+      </c>
+      <c r="H2723">
+        <v>0</v>
+      </c>
+      <c r="L2723">
+        <v>11.3</v>
+      </c>
+      <c r="M2723">
+        <v>103.9</v>
+      </c>
+      <c r="N2723">
+        <v>0.67</v>
+      </c>
+      <c r="O2723">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="2724" spans="2:15">
+      <c r="D2724">
+        <v>2</v>
+      </c>
+      <c r="F2724">
+        <v>0.1</v>
+      </c>
+      <c r="G2724">
+        <v>0</v>
+      </c>
+      <c r="H2724">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2725" spans="2:15">
+      <c r="D2725">
+        <v>3</v>
+      </c>
+      <c r="F2725">
+        <v>0.1</v>
+      </c>
+      <c r="G2725">
+        <v>0</v>
+      </c>
+      <c r="H2725">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2726" spans="2:15">
+      <c r="B2726" s="1">
+        <v>0.61805555555555558</v>
+      </c>
+      <c r="C2726" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D2726">
+        <v>1</v>
+      </c>
+      <c r="F2726">
+        <v>0.1</v>
+      </c>
+      <c r="G2726">
+        <v>0</v>
+      </c>
+      <c r="H2726">
+        <v>0</v>
+      </c>
+      <c r="L2726">
+        <v>12.9</v>
+      </c>
+      <c r="M2726">
+        <v>100.4</v>
+      </c>
+      <c r="N2726">
+        <v>0.23</v>
+      </c>
+      <c r="O2726">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="2727" spans="2:15">
+      <c r="D2727">
+        <v>2</v>
+      </c>
+      <c r="F2727">
+        <v>0.1</v>
+      </c>
+      <c r="G2727">
+        <v>0</v>
+      </c>
+      <c r="H2727">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2728" spans="2:15">
+      <c r="D2728">
+        <v>3</v>
+      </c>
+      <c r="F2728">
+        <v>0.1</v>
+      </c>
+      <c r="G2728">
+        <v>0</v>
+      </c>
+      <c r="H2728">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2729" spans="2:15">
+      <c r="B2729" s="1">
+        <v>0.63402777777777775</v>
+      </c>
+      <c r="C2729" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D2729">
+        <v>1</v>
+      </c>
+      <c r="F2729">
+        <v>0.1</v>
+      </c>
+      <c r="G2729">
+        <v>0</v>
+      </c>
+      <c r="H2729">
+        <v>0</v>
+      </c>
+      <c r="L2729">
+        <v>11.6</v>
+      </c>
+      <c r="M2729">
+        <v>96.7</v>
+      </c>
+      <c r="N2729">
+        <v>1.28</v>
+      </c>
+      <c r="O2729">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="2730" spans="2:15">
+      <c r="D2730">
+        <v>2</v>
+      </c>
+      <c r="F2730">
+        <v>0.1</v>
+      </c>
+      <c r="G2730">
+        <v>0</v>
+      </c>
+      <c r="H2730">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2731" spans="2:15">
+      <c r="D2731">
+        <v>3</v>
+      </c>
+      <c r="F2731">
+        <v>0.1</v>
+      </c>
+      <c r="G2731">
+        <v>0</v>
+      </c>
+      <c r="H2731">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2732" spans="2:15">
+      <c r="B2732" s="1">
+        <v>0.65</v>
+      </c>
+      <c r="C2732" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="D2732">
+        <v>1</v>
+      </c>
+      <c r="F2732">
+        <v>0.1</v>
+      </c>
+      <c r="G2732">
+        <v>10.78</v>
+      </c>
+      <c r="H2732">
+        <v>0</v>
+      </c>
+      <c r="L2732">
+        <v>12.6</v>
+      </c>
+      <c r="M2732">
+        <v>101.4</v>
+      </c>
+      <c r="N2732">
+        <v>3.71</v>
+      </c>
+      <c r="O2732">
+        <v>2.68</v>
+      </c>
+    </row>
+    <row r="2733" spans="2:15">
+      <c r="D2733">
+        <v>2</v>
+      </c>
+      <c r="F2733">
+        <v>0</v>
+      </c>
+      <c r="G2733">
+        <v>9.01</v>
+      </c>
+      <c r="H2733">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="2734" spans="2:15">
+      <c r="D2734">
+        <v>3</v>
+      </c>
+      <c r="F2734">
+        <v>0.1</v>
+      </c>
+      <c r="G2734">
+        <v>3.01</v>
+      </c>
+      <c r="H2734">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="2735" spans="2:15">
+      <c r="B2735" s="1">
+        <v>0.66319444444444442</v>
+      </c>
+      <c r="C2735" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="D2735">
+        <v>1</v>
+      </c>
+      <c r="F2735">
+        <v>0.1</v>
+      </c>
+      <c r="G2735">
+        <v>1.04</v>
+      </c>
+      <c r="H2735">
+        <v>0.09</v>
+      </c>
+      <c r="L2735">
+        <v>13.9</v>
+      </c>
+      <c r="M2735">
+        <v>98.9</v>
+      </c>
+      <c r="N2735">
+        <v>2.31</v>
+      </c>
+      <c r="O2735">
+        <v>1.69</v>
+      </c>
+    </row>
+    <row r="2736" spans="2:15">
+      <c r="C2736" s="3"/>
+      <c r="D2736">
+        <v>2</v>
+      </c>
+      <c r="F2736">
+        <v>0.1</v>
+      </c>
+      <c r="G2736">
+        <v>5.37</v>
+      </c>
+      <c r="H2736">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="2737" spans="1:15">
+      <c r="D2737">
+        <v>3</v>
+      </c>
+      <c r="F2737">
+        <v>0.1</v>
+      </c>
+      <c r="G2737">
+        <v>7.44</v>
+      </c>
+      <c r="H2737">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="2738" spans="1:15" s="19" customFormat="1">
+      <c r="E2738" s="36"/>
+    </row>
+    <row r="2739" spans="1:15">
+      <c r="A2739" t="s">
+        <v>392</v>
+      </c>
+      <c r="B2739" s="1">
+        <v>0.57152777777777775</v>
+      </c>
+      <c r="C2739" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2739">
+        <v>1</v>
+      </c>
+      <c r="F2739">
+        <v>0.1</v>
+      </c>
+      <c r="G2739">
+        <v>2.27</v>
+      </c>
+      <c r="H2739">
+        <v>0.04</v>
+      </c>
+      <c r="L2739">
+        <v>13.1</v>
+      </c>
+      <c r="M2739">
+        <v>96.8</v>
+      </c>
+      <c r="N2739">
+        <v>13.21</v>
+      </c>
+      <c r="O2739">
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="2740" spans="1:15">
+      <c r="D2740">
+        <v>2</v>
+      </c>
+      <c r="F2740">
+        <v>0.1</v>
+      </c>
+      <c r="G2740">
+        <v>1.73</v>
+      </c>
+      <c r="H2740">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="2741" spans="1:15">
+      <c r="D2741">
+        <v>3</v>
+      </c>
+      <c r="F2741">
+        <v>0.1</v>
+      </c>
+      <c r="G2741">
+        <v>2.81</v>
+      </c>
+      <c r="H2741">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="2742" spans="1:15">
+      <c r="B2742" s="1">
+        <v>0.55277777777777781</v>
+      </c>
+      <c r="C2742" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2742">
+        <v>1</v>
+      </c>
+      <c r="F2742">
+        <v>0.1</v>
+      </c>
+      <c r="G2742">
+        <v>1.39</v>
+      </c>
+      <c r="H2742">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="L2742">
+        <v>12.9</v>
+      </c>
+      <c r="M2742">
+        <v>95.4</v>
+      </c>
+      <c r="N2742">
+        <v>21.71</v>
+      </c>
+      <c r="O2742">
+        <v>1.48</v>
+      </c>
+    </row>
+    <row r="2743" spans="1:15">
+      <c r="D2743">
+        <v>2</v>
+      </c>
+      <c r="F2743">
+        <v>0.1</v>
+      </c>
+      <c r="G2743">
+        <v>1.04</v>
+      </c>
+      <c r="H2743">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="2744" spans="1:15">
+      <c r="D2744">
+        <v>3</v>
+      </c>
+      <c r="F2744">
+        <v>0.1</v>
+      </c>
+      <c r="G2744">
+        <v>2.27</v>
+      </c>
+      <c r="H2744">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="2745" spans="1:15">
+      <c r="B2745" s="1">
+        <v>0.53541666666666665</v>
+      </c>
+      <c r="C2745" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D2745">
+        <v>1</v>
+      </c>
+      <c r="F2745">
+        <v>19.39</v>
+      </c>
+      <c r="G2745">
+        <v>0</v>
+      </c>
+      <c r="H2745">
+        <v>0</v>
+      </c>
+      <c r="L2745">
+        <v>11.8</v>
+      </c>
+      <c r="M2745">
+        <v>93.9</v>
+      </c>
+      <c r="N2745">
+        <v>13.29</v>
+      </c>
+      <c r="O2745">
+        <v>1.1000000000000001</v>
+      </c>
+    </row>
+    <row r="2746" spans="1:15">
+      <c r="D2746">
+        <v>2</v>
+      </c>
+      <c r="F2746">
+        <v>6.25</v>
+      </c>
+      <c r="G2746">
+        <v>0</v>
+      </c>
+      <c r="H2746">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2747" spans="1:15">
+      <c r="D2747">
+        <v>3</v>
+      </c>
+      <c r="F2747">
+        <v>0.1</v>
+      </c>
+      <c r="G2747">
+        <v>1</v>
+      </c>
+      <c r="H2747">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="2748" spans="1:15">
+      <c r="B2748" s="1">
+        <v>0.52013888888888893</v>
+      </c>
+      <c r="C2748" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D2748">
+        <v>1</v>
+      </c>
+      <c r="F2748">
+        <v>6.25</v>
+      </c>
+      <c r="G2748">
+        <v>3.01</v>
+      </c>
+      <c r="H2748">
+        <v>2.0699999999999998</v>
+      </c>
+      <c r="L2748">
+        <v>12.2</v>
+      </c>
+      <c r="M2748">
+        <v>88.4</v>
+      </c>
+      <c r="N2748">
+        <v>76.72</v>
+      </c>
+      <c r="O2748">
+        <v>9.84</v>
+      </c>
+    </row>
+    <row r="2749" spans="1:15">
+      <c r="D2749">
+        <v>2</v>
+      </c>
+      <c r="F2749">
+        <v>35.82</v>
+      </c>
+      <c r="G2749">
+        <v>1.34</v>
+      </c>
+      <c r="H2749">
+        <v>26.73</v>
+      </c>
+    </row>
+    <row r="2750" spans="1:15">
+      <c r="D2750">
+        <v>3</v>
+      </c>
+      <c r="F2750">
+        <v>96.08</v>
+      </c>
+      <c r="G2750">
+        <v>4.63</v>
+      </c>
+      <c r="H2750">
+        <v>20.75</v>
+      </c>
+    </row>
+    <row r="2751" spans="1:15">
+      <c r="B2751" s="1">
+        <v>0.48888888888888887</v>
+      </c>
+      <c r="C2751" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D2751">
+        <v>1</v>
+      </c>
+      <c r="F2751">
+        <v>0.1</v>
+      </c>
+      <c r="G2751">
+        <v>0.05</v>
+      </c>
+      <c r="H2751">
+        <v>2</v>
+      </c>
+      <c r="L2751">
+        <v>12.6</v>
+      </c>
+      <c r="M2751">
+        <v>96.1</v>
+      </c>
+      <c r="N2751">
+        <v>7.11</v>
+      </c>
+      <c r="O2751">
+        <v>3.56</v>
+      </c>
+    </row>
+    <row r="2752" spans="1:15">
+      <c r="D2752">
+        <v>2</v>
+      </c>
+      <c r="F2752">
+        <v>0.1</v>
+      </c>
+      <c r="G2752">
+        <v>2.77</v>
+      </c>
+      <c r="H2752">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="2753" spans="2:15">
+      <c r="D2753">
+        <v>3</v>
+      </c>
+      <c r="F2753">
+        <v>0.1</v>
+      </c>
+      <c r="G2753">
+        <v>3.95</v>
+      </c>
+      <c r="H2753">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="2754" spans="2:15">
+      <c r="B2754" s="1">
+        <v>0.4826388888888889</v>
+      </c>
+      <c r="C2754" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D2754">
+        <v>1</v>
+      </c>
+      <c r="F2754">
+        <v>0.1</v>
+      </c>
+      <c r="G2754">
+        <v>0.05</v>
+      </c>
+      <c r="H2754">
+        <v>2</v>
+      </c>
+      <c r="L2754">
+        <v>12.2</v>
+      </c>
+      <c r="M2754">
+        <v>99.2</v>
+      </c>
+      <c r="N2754">
+        <v>0.85</v>
+      </c>
+      <c r="O2754">
+        <v>0.26</v>
+      </c>
+    </row>
+    <row r="2755" spans="2:15">
+      <c r="D2755">
+        <v>2</v>
+      </c>
+      <c r="F2755">
+        <v>7.75</v>
+      </c>
+      <c r="G2755">
+        <v>0.6</v>
+      </c>
+      <c r="H2755">
+        <v>12.91</v>
+      </c>
+    </row>
+    <row r="2756" spans="2:15">
+      <c r="D2756">
+        <v>3</v>
+      </c>
+      <c r="F2756">
+        <v>20.170000000000002</v>
+      </c>
+      <c r="G2756">
+        <v>0.75</v>
+      </c>
+      <c r="H2756">
+        <v>26.89</v>
+      </c>
+    </row>
+    <row r="2757" spans="2:15">
+      <c r="B2757" s="1">
+        <v>0.47569444444444442</v>
+      </c>
+      <c r="C2757" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D2757">
+        <v>1</v>
+      </c>
+      <c r="F2757">
+        <v>20.95</v>
+      </c>
+      <c r="G2757">
+        <v>0.8</v>
+      </c>
+      <c r="H2757">
+        <v>26.18</v>
+      </c>
+      <c r="L2757">
+        <v>12.4</v>
+      </c>
+      <c r="M2757">
+        <v>98.6</v>
+      </c>
+      <c r="N2757">
+        <v>0.71</v>
+      </c>
+      <c r="O2757">
+        <v>0.42</v>
+      </c>
+    </row>
+    <row r="2758" spans="2:15">
+      <c r="D2758">
+        <v>2</v>
+      </c>
+      <c r="F2758">
+        <v>79.650000000000006</v>
+      </c>
+      <c r="G2758">
+        <v>1.29</v>
+      </c>
+      <c r="H2758">
+        <v>61.74</v>
+      </c>
+    </row>
+    <row r="2759" spans="2:15">
+      <c r="D2759">
+        <v>3</v>
+      </c>
+      <c r="F2759">
+        <v>25.65</v>
+      </c>
+      <c r="G2759">
+        <v>1.04</v>
+      </c>
+      <c r="H2759">
+        <v>24.66</v>
+      </c>
+    </row>
+    <row r="2760" spans="2:15">
+      <c r="B2760" s="1">
+        <v>0.41041666666666665</v>
+      </c>
+      <c r="C2760" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D2760">
+        <v>1</v>
+      </c>
+      <c r="F2760">
+        <v>34.25</v>
+      </c>
+      <c r="G2760">
+        <v>0.95</v>
+      </c>
+      <c r="H2760">
+        <v>36.06</v>
+      </c>
+      <c r="L2760">
+        <v>11</v>
+      </c>
+      <c r="M2760">
+        <v>97.3</v>
+      </c>
+      <c r="N2760">
+        <v>0.92</v>
+      </c>
+      <c r="O2760">
+        <v>0.21</v>
+      </c>
+    </row>
+    <row r="2761" spans="2:15">
+      <c r="D2761">
+        <v>2</v>
+      </c>
+      <c r="F2761">
+        <v>7.75</v>
+      </c>
+      <c r="G2761">
+        <v>0.4</v>
+      </c>
+      <c r="H2761">
+        <v>19.37</v>
+      </c>
+    </row>
+    <row r="2762" spans="2:15">
+      <c r="D2762">
+        <v>3</v>
+      </c>
+      <c r="F2762">
+        <v>40.520000000000003</v>
+      </c>
+      <c r="G2762">
+        <v>1.29</v>
+      </c>
+      <c r="H2762">
+        <v>31.41</v>
+      </c>
+    </row>
+    <row r="2763" spans="2:15">
+      <c r="B2763" s="1">
+        <v>0.4548611111111111</v>
+      </c>
+      <c r="C2763" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="D2763">
+        <v>1</v>
+      </c>
+      <c r="F2763">
+        <v>0.1</v>
+      </c>
+      <c r="G2763">
+        <v>0.3</v>
+      </c>
+      <c r="H2763">
+        <v>0.33</v>
+      </c>
+      <c r="L2763">
+        <v>12.2</v>
+      </c>
+      <c r="M2763">
+        <v>98.7</v>
+      </c>
+      <c r="N2763">
+        <v>0.81</v>
+      </c>
+      <c r="O2763">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="2764" spans="2:15">
+      <c r="D2764">
+        <v>2</v>
+      </c>
+      <c r="F2764">
+        <v>36.6</v>
+      </c>
+      <c r="G2764">
+        <v>0.75</v>
+      </c>
+      <c r="H2764">
+        <v>48.8</v>
+      </c>
+    </row>
+    <row r="2765" spans="2:15">
+      <c r="D2765">
+        <v>3</v>
+      </c>
+      <c r="F2765">
+        <v>39.729999999999997</v>
+      </c>
+      <c r="G2765">
+        <v>0.85</v>
+      </c>
+      <c r="H2765">
+        <v>46.74</v>
+      </c>
+    </row>
+    <row r="2766" spans="2:15">
+      <c r="B2766" s="1">
+        <v>0.58888888888888891</v>
+      </c>
+      <c r="C2766" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="D2766">
+        <v>1</v>
+      </c>
+      <c r="F2766">
+        <v>0.1</v>
+      </c>
+      <c r="G2766">
+        <v>1.63</v>
+      </c>
+      <c r="H2766">
+        <v>0.06</v>
+      </c>
+      <c r="L2766">
+        <v>15.3</v>
+      </c>
+      <c r="M2766">
+        <v>97.6</v>
+      </c>
+      <c r="N2766">
+        <v>0.84</v>
+      </c>
+      <c r="O2766">
+        <v>0.66</v>
+      </c>
+    </row>
+    <row r="2767" spans="2:15">
+      <c r="C2767" s="3"/>
+      <c r="D2767">
+        <v>2</v>
+      </c>
+      <c r="F2767">
+        <v>0.1</v>
+      </c>
+      <c r="G2767">
+        <v>1.0900000000000001</v>
+      </c>
+      <c r="H2767">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="2768" spans="2:15">
+      <c r="D2768">
+        <v>3</v>
+      </c>
+      <c r="F2768">
+        <v>0.1</v>
+      </c>
+      <c r="G2768">
+        <v>1.73</v>
+      </c>
+      <c r="H2768">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="2769" spans="5:5" s="19" customFormat="1">
+      <c r="E2769" s="36"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
local commit of talt cyano data
</commit_message>
<xml_diff>
--- a/data/talt_cyano/talt_cyano_digitized.xlsx
+++ b/data/talt_cyano/talt_cyano_digitized.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29212"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29225"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="20435" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ED0097AE-E8BF-4194-85E9-A632FE632A20}"/>
+  <xr:revisionPtr revIDLastSave="20831" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CE9692C1-B11D-466F-9214-9CC4539DAEFC}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1854" uniqueCount="390">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1878" uniqueCount="393">
   <si>
     <t>Date</t>
   </si>
@@ -1197,10 +1197,19 @@
     <t xml:space="preserve">18/08/2025 </t>
   </si>
   <si>
+    <t xml:space="preserve">0.34	</t>
+  </si>
+  <si>
     <t xml:space="preserve">20/08/2025 </t>
   </si>
   <si>
     <t xml:space="preserve">22/08/2025 </t>
+  </si>
+  <si>
+    <t>25/08/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">29/08/2025 </t>
   </si>
 </sst>
 </file>
@@ -1758,7 +1767,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S2707"/>
+  <dimension ref="A1:S2769"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="11.7109375" customWidth="1"/>
@@ -68701,6 +68710,9 @@
       <c r="A2615" t="s">
         <v>387</v>
       </c>
+      <c r="B2615" s="1">
+        <v>0.43541666666666667</v>
+      </c>
       <c r="C2615" s="3" t="s">
         <v>20</v>
       </c>
@@ -68719,6 +68731,18 @@
       <c r="H2615">
         <v>0</v>
       </c>
+      <c r="L2615">
+        <v>11.3</v>
+      </c>
+      <c r="M2615">
+        <v>98.4</v>
+      </c>
+      <c r="N2615">
+        <v>1.01</v>
+      </c>
+      <c r="O2615" t="s">
+        <v>388</v>
+      </c>
       <c r="P2615" t="s">
         <v>319</v>
       </c>
@@ -68752,6 +68776,9 @@
       </c>
     </row>
     <row r="2618" spans="1:18">
+      <c r="B2618" s="1">
+        <v>0.45694444444444443</v>
+      </c>
       <c r="C2618" s="3" t="s">
         <v>25</v>
       </c>
@@ -68767,6 +68794,18 @@
       <c r="H2618">
         <v>0</v>
       </c>
+      <c r="L2618">
+        <v>12.6</v>
+      </c>
+      <c r="M2618">
+        <v>88.4</v>
+      </c>
+      <c r="N2618">
+        <v>2.84</v>
+      </c>
+      <c r="O2618">
+        <v>0.17</v>
+      </c>
     </row>
     <row r="2619" spans="1:18">
       <c r="D2619">
@@ -68797,6 +68836,9 @@
       </c>
     </row>
     <row r="2621" spans="1:18">
+      <c r="B2621" s="1">
+        <v>0.47430555555555554</v>
+      </c>
       <c r="C2621" s="3" t="s">
         <v>27</v>
       </c>
@@ -68812,6 +68854,18 @@
       <c r="H2621">
         <v>0.09</v>
       </c>
+      <c r="L2621">
+        <v>11.3</v>
+      </c>
+      <c r="M2621">
+        <v>99</v>
+      </c>
+      <c r="N2621">
+        <v>2.12</v>
+      </c>
+      <c r="O2621">
+        <v>0.22</v>
+      </c>
     </row>
     <row r="2622" spans="1:18">
       <c r="D2622">
@@ -68842,6 +68896,9 @@
       </c>
     </row>
     <row r="2624" spans="1:18">
+      <c r="B2624" s="1">
+        <v>0.49236111111111114</v>
+      </c>
       <c r="C2624" s="3" t="s">
         <v>58</v>
       </c>
@@ -68857,8 +68914,20 @@
       <c r="H2624">
         <v>2</v>
       </c>
-    </row>
-    <row r="2625" spans="3:8">
+      <c r="L2624">
+        <v>11.7</v>
+      </c>
+      <c r="M2624">
+        <v>90.6</v>
+      </c>
+      <c r="N2624">
+        <v>7.08</v>
+      </c>
+      <c r="O2624">
+        <v>4.43</v>
+      </c>
+    </row>
+    <row r="2625" spans="2:15">
       <c r="D2625">
         <v>2</v>
       </c>
@@ -68872,7 +68941,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2626" spans="3:8">
+    <row r="2626" spans="2:15">
       <c r="D2626">
         <v>3</v>
       </c>
@@ -68886,7 +68955,10 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="2627" spans="3:8">
+    <row r="2627" spans="2:15">
+      <c r="B2627" s="1">
+        <v>0.50694444444444442</v>
+      </c>
       <c r="C2627" s="3" t="s">
         <v>29</v>
       </c>
@@ -68902,8 +68974,20 @@
       <c r="H2627">
         <v>0</v>
       </c>
-    </row>
-    <row r="2628" spans="3:8">
+      <c r="L2627">
+        <v>11.8</v>
+      </c>
+      <c r="M2627">
+        <v>111.2</v>
+      </c>
+      <c r="N2627">
+        <v>0.86</v>
+      </c>
+      <c r="O2627">
+        <v>0.17</v>
+      </c>
+    </row>
+    <row r="2628" spans="2:15">
       <c r="D2628">
         <v>2</v>
       </c>
@@ -68917,7 +69001,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2629" spans="3:8">
+    <row r="2629" spans="2:15">
       <c r="D2629">
         <v>3</v>
       </c>
@@ -68931,7 +69015,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2630" spans="3:8">
+    <row r="2630" spans="2:15">
+      <c r="B2630" s="1">
+        <v>0.51597222222222228</v>
+      </c>
       <c r="C2630" s="3" t="s">
         <v>30</v>
       </c>
@@ -68947,8 +69034,20 @@
       <c r="H2630">
         <v>0</v>
       </c>
-    </row>
-    <row r="2631" spans="3:8">
+      <c r="L2630">
+        <v>11.9</v>
+      </c>
+      <c r="M2630">
+        <v>105</v>
+      </c>
+      <c r="N2630">
+        <v>0.54</v>
+      </c>
+      <c r="O2630">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="2631" spans="2:15">
       <c r="D2631">
         <v>2</v>
       </c>
@@ -68962,7 +69061,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2632" spans="3:8">
+    <row r="2632" spans="2:15">
       <c r="D2632">
         <v>3</v>
       </c>
@@ -68976,7 +69075,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2633" spans="3:8">
+    <row r="2633" spans="2:15">
+      <c r="B2633" s="1">
+        <v>0.52916666666666667</v>
+      </c>
       <c r="C2633" s="3" t="s">
         <v>31</v>
       </c>
@@ -68992,8 +69094,20 @@
       <c r="H2633">
         <v>0</v>
       </c>
-    </row>
-    <row r="2634" spans="3:8">
+      <c r="L2633">
+        <v>12.3</v>
+      </c>
+      <c r="M2633">
+        <v>102.9</v>
+      </c>
+      <c r="N2633">
+        <v>0.31</v>
+      </c>
+      <c r="O2633">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="2634" spans="2:15">
       <c r="D2634">
         <v>2</v>
       </c>
@@ -69007,7 +69121,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2635" spans="3:8">
+    <row r="2635" spans="2:15">
       <c r="D2635">
         <v>3</v>
       </c>
@@ -69021,7 +69135,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2636" spans="3:8">
+    <row r="2636" spans="2:15">
+      <c r="B2636" s="1">
+        <v>0.54305555555555551</v>
+      </c>
       <c r="C2636" s="3" t="s">
         <v>32</v>
       </c>
@@ -69037,8 +69154,20 @@
       <c r="H2636">
         <v>0.03</v>
       </c>
-    </row>
-    <row r="2637" spans="3:8">
+      <c r="L2636">
+        <v>11.9</v>
+      </c>
+      <c r="M2636">
+        <v>100.4</v>
+      </c>
+      <c r="N2636">
+        <v>0.87</v>
+      </c>
+      <c r="O2636">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="2637" spans="2:15">
       <c r="D2637">
         <v>2</v>
       </c>
@@ -69052,7 +69181,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2638" spans="3:8">
+    <row r="2638" spans="2:15">
       <c r="D2638">
         <v>3</v>
       </c>
@@ -69066,7 +69195,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2639" spans="3:8">
+    <row r="2639" spans="2:15">
+      <c r="B2639" s="1">
+        <v>0.56666666666666665</v>
+      </c>
       <c r="C2639" s="3" t="s">
         <v>41</v>
       </c>
@@ -69082,8 +69214,20 @@
       <c r="H2639">
         <v>0</v>
       </c>
-    </row>
-    <row r="2640" spans="3:8">
+      <c r="L2639">
+        <v>12.5</v>
+      </c>
+      <c r="M2639">
+        <v>103.4</v>
+      </c>
+      <c r="N2639">
+        <v>1.34</v>
+      </c>
+      <c r="O2639">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="2640" spans="2:15">
       <c r="D2640">
         <v>2</v>
       </c>
@@ -69112,6 +69256,9 @@
       </c>
     </row>
     <row r="2642" spans="1:16">
+      <c r="B2642" s="1">
+        <v>0.5756944444444444</v>
+      </c>
       <c r="C2642" s="3" t="s">
         <v>34</v>
       </c>
@@ -69126,6 +69273,18 @@
       </c>
       <c r="H2642">
         <v>0</v>
+      </c>
+      <c r="L2642">
+        <v>13.2</v>
+      </c>
+      <c r="M2642">
+        <v>94.1</v>
+      </c>
+      <c r="N2642">
+        <v>2.4700000000000002</v>
+      </c>
+      <c r="O2642">
+        <v>0.27</v>
       </c>
     </row>
     <row r="2643" spans="1:16">
@@ -69162,7 +69321,10 @@
     </row>
     <row r="2646" spans="1:16">
       <c r="A2646" t="s">
-        <v>388</v>
+        <v>389</v>
+      </c>
+      <c r="B2646" s="1">
+        <v>0.48958333333333331</v>
       </c>
       <c r="C2646" s="3" t="s">
         <v>20</v>
@@ -69182,6 +69344,18 @@
       <c r="H2646">
         <v>0</v>
       </c>
+      <c r="L2646">
+        <v>10.8</v>
+      </c>
+      <c r="M2646">
+        <v>90.6</v>
+      </c>
+      <c r="N2646">
+        <v>4.1500000000000004</v>
+      </c>
+      <c r="O2646">
+        <v>0.08</v>
+      </c>
       <c r="P2646" t="s">
         <v>147</v>
       </c>
@@ -69215,6 +69389,9 @@
       </c>
     </row>
     <row r="2649" spans="1:16">
+      <c r="B2649" s="1">
+        <v>0.50069444444444444</v>
+      </c>
       <c r="C2649" s="3" t="s">
         <v>25</v>
       </c>
@@ -69230,6 +69407,18 @@
       <c r="H2649">
         <v>0</v>
       </c>
+      <c r="L2649">
+        <v>10.8</v>
+      </c>
+      <c r="M2649">
+        <v>95.8</v>
+      </c>
+      <c r="N2649">
+        <v>4.93</v>
+      </c>
+      <c r="O2649">
+        <v>0.15</v>
+      </c>
     </row>
     <row r="2650" spans="1:16">
       <c r="D2650">
@@ -69260,6 +69449,9 @@
       </c>
     </row>
     <row r="2652" spans="1:16">
+      <c r="B2652" s="1">
+        <v>0.51597222222222228</v>
+      </c>
       <c r="C2652" s="3" t="s">
         <v>27</v>
       </c>
@@ -69275,6 +69467,18 @@
       <c r="H2652">
         <v>0</v>
       </c>
+      <c r="L2652">
+        <v>9.9</v>
+      </c>
+      <c r="M2652">
+        <v>97.1</v>
+      </c>
+      <c r="N2652">
+        <v>10.51</v>
+      </c>
+      <c r="O2652">
+        <v>0.28000000000000003</v>
+      </c>
     </row>
     <row r="2653" spans="1:16">
       <c r="D2653">
@@ -69305,6 +69509,9 @@
       </c>
     </row>
     <row r="2655" spans="1:16">
+      <c r="B2655" s="1">
+        <v>0.52569444444444446</v>
+      </c>
       <c r="C2655" s="3" t="s">
         <v>58</v>
       </c>
@@ -69320,6 +69527,18 @@
       <c r="H2655">
         <v>0.15</v>
       </c>
+      <c r="L2655">
+        <v>9.3000000000000007</v>
+      </c>
+      <c r="M2655">
+        <v>99.3</v>
+      </c>
+      <c r="N2655">
+        <v>13.22</v>
+      </c>
+      <c r="O2655">
+        <v>0.91</v>
+      </c>
     </row>
     <row r="2656" spans="1:16">
       <c r="D2656">
@@ -69335,7 +69554,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2657" spans="3:8">
+    <row r="2657" spans="2:15">
       <c r="D2657">
         <v>3</v>
       </c>
@@ -69349,7 +69568,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2658" spans="3:8">
+    <row r="2658" spans="2:15">
+      <c r="B2658" s="1">
+        <v>0.53611111111111109</v>
+      </c>
       <c r="C2658" s="3" t="s">
         <v>29</v>
       </c>
@@ -69365,8 +69587,20 @@
       <c r="H2658">
         <v>7.0000000000000007E-2</v>
       </c>
-    </row>
-    <row r="2659" spans="3:8">
+      <c r="L2658">
+        <v>9.3000000000000007</v>
+      </c>
+      <c r="M2658">
+        <v>101.3</v>
+      </c>
+      <c r="N2658">
+        <v>15.49</v>
+      </c>
+      <c r="O2658">
+        <v>2.31</v>
+      </c>
+    </row>
+    <row r="2659" spans="2:15">
       <c r="D2659">
         <v>2</v>
       </c>
@@ -69380,7 +69614,7 @@
         <v>0.08</v>
       </c>
     </row>
-    <row r="2660" spans="3:8">
+    <row r="2660" spans="2:15">
       <c r="D2660">
         <v>3</v>
       </c>
@@ -69394,7 +69628,10 @@
         <v>0.08</v>
       </c>
     </row>
-    <row r="2661" spans="3:8">
+    <row r="2661" spans="2:15">
+      <c r="B2661" s="1">
+        <v>0.54652777777777772</v>
+      </c>
       <c r="C2661" s="3" t="s">
         <v>30</v>
       </c>
@@ -69410,8 +69647,20 @@
       <c r="H2661">
         <v>18.75</v>
       </c>
-    </row>
-    <row r="2662" spans="3:8">
+      <c r="L2661">
+        <v>9.3000000000000007</v>
+      </c>
+      <c r="M2661">
+        <v>96.7</v>
+      </c>
+      <c r="N2661">
+        <v>20.260000000000002</v>
+      </c>
+      <c r="O2661">
+        <v>3.07</v>
+      </c>
+    </row>
+    <row r="2662" spans="2:15">
       <c r="D2662">
         <v>2</v>
       </c>
@@ -69425,7 +69674,7 @@
         <v>9.0500000000000007</v>
       </c>
     </row>
-    <row r="2663" spans="3:8">
+    <row r="2663" spans="2:15">
       <c r="D2663">
         <v>3</v>
       </c>
@@ -69439,7 +69688,10 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="2664" spans="3:8">
+    <row r="2664" spans="2:15">
+      <c r="B2664" s="1">
+        <v>0.5541666666666667</v>
+      </c>
       <c r="C2664" s="3" t="s">
         <v>31</v>
       </c>
@@ -69455,8 +69707,20 @@
       <c r="H2664">
         <v>0</v>
       </c>
-    </row>
-    <row r="2665" spans="3:8">
+      <c r="L2664">
+        <v>12.6</v>
+      </c>
+      <c r="M2664">
+        <v>102.8</v>
+      </c>
+      <c r="N2664">
+        <v>3.31</v>
+      </c>
+      <c r="O2664">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="2665" spans="2:15">
       <c r="D2665">
         <v>2</v>
       </c>
@@ -69470,7 +69734,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2666" spans="3:8">
+    <row r="2666" spans="2:15">
       <c r="D2666">
         <v>3</v>
       </c>
@@ -69484,7 +69748,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2667" spans="3:8">
+    <row r="2667" spans="2:15">
+      <c r="B2667" s="1">
+        <v>0.56111111111111112</v>
+      </c>
       <c r="C2667" s="3" t="s">
         <v>32</v>
       </c>
@@ -69500,8 +69767,20 @@
       <c r="H2667">
         <v>0</v>
       </c>
-    </row>
-    <row r="2668" spans="3:8">
+      <c r="L2667">
+        <v>10.4</v>
+      </c>
+      <c r="M2667">
+        <v>98.8</v>
+      </c>
+      <c r="N2667">
+        <v>9.1199999999999992</v>
+      </c>
+      <c r="O2667">
+        <v>0.32</v>
+      </c>
+    </row>
+    <row r="2668" spans="2:15">
       <c r="D2668">
         <v>2</v>
       </c>
@@ -69515,7 +69794,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2669" spans="3:8">
+    <row r="2669" spans="2:15">
       <c r="D2669">
         <v>3</v>
       </c>
@@ -69529,7 +69808,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2670" spans="3:8">
+    <row r="2670" spans="2:15">
+      <c r="B2670" s="1">
+        <v>0.57708333333333328</v>
+      </c>
       <c r="C2670" s="3" t="s">
         <v>41</v>
       </c>
@@ -69545,8 +69827,20 @@
       <c r="H2670">
         <v>0</v>
       </c>
-    </row>
-    <row r="2671" spans="3:8">
+      <c r="L2670">
+        <v>11.5</v>
+      </c>
+      <c r="M2670">
+        <v>105.1</v>
+      </c>
+      <c r="N2670">
+        <v>1.66</v>
+      </c>
+      <c r="O2670">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="2671" spans="2:15">
       <c r="D2671">
         <v>2</v>
       </c>
@@ -69560,7 +69854,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2672" spans="3:8">
+    <row r="2672" spans="2:15">
       <c r="D2672">
         <v>3</v>
       </c>
@@ -69575,6 +69869,9 @@
       </c>
     </row>
     <row r="2673" spans="1:16">
+      <c r="B2673" s="1">
+        <v>0.58333333333333337</v>
+      </c>
       <c r="C2673" s="3" t="s">
         <v>34</v>
       </c>
@@ -69589,6 +69886,18 @@
       </c>
       <c r="H2673">
         <v>0</v>
+      </c>
+      <c r="L2673">
+        <v>11</v>
+      </c>
+      <c r="M2673">
+        <v>96.6</v>
+      </c>
+      <c r="N2673">
+        <v>1.94</v>
+      </c>
+      <c r="O2673">
+        <v>0.04</v>
       </c>
     </row>
     <row r="2674" spans="1:16">
@@ -69625,7 +69934,10 @@
     </row>
     <row r="2677" spans="1:16">
       <c r="A2677" t="s">
-        <v>389</v>
+        <v>390</v>
+      </c>
+      <c r="B2677" s="1">
+        <v>0.50069444444444444</v>
       </c>
       <c r="C2677" s="3" t="s">
         <v>20</v>
@@ -69645,6 +69957,18 @@
       <c r="H2677">
         <v>0</v>
       </c>
+      <c r="L2677">
+        <v>12.2</v>
+      </c>
+      <c r="M2677">
+        <v>95.7</v>
+      </c>
+      <c r="N2677">
+        <v>1.1399999999999999</v>
+      </c>
+      <c r="O2677">
+        <v>0.08</v>
+      </c>
       <c r="P2677" t="s">
         <v>157</v>
       </c>
@@ -69678,6 +70002,9 @@
       </c>
     </row>
     <row r="2680" spans="1:16">
+      <c r="B2680" s="1">
+        <v>0.5180555555555556</v>
+      </c>
       <c r="C2680" s="3" t="s">
         <v>25</v>
       </c>
@@ -69693,6 +70020,18 @@
       <c r="H2680">
         <v>0</v>
       </c>
+      <c r="L2680">
+        <v>11.3</v>
+      </c>
+      <c r="M2680">
+        <v>100.3</v>
+      </c>
+      <c r="N2680">
+        <v>1.94</v>
+      </c>
+      <c r="O2680">
+        <v>0.15</v>
+      </c>
     </row>
     <row r="2681" spans="1:16">
       <c r="D2681">
@@ -69723,6 +70062,9 @@
       </c>
     </row>
     <row r="2683" spans="1:16">
+      <c r="B2683" s="1">
+        <v>0.57152777777777775</v>
+      </c>
       <c r="C2683" s="3" t="s">
         <v>27</v>
       </c>
@@ -69738,6 +70080,18 @@
       <c r="H2683">
         <v>0</v>
       </c>
+      <c r="L2683">
+        <v>11.5</v>
+      </c>
+      <c r="M2683">
+        <v>92.8</v>
+      </c>
+      <c r="N2683">
+        <v>1.75</v>
+      </c>
+      <c r="O2683">
+        <v>0.06</v>
+      </c>
     </row>
     <row r="2684" spans="1:16">
       <c r="D2684">
@@ -69768,6 +70122,9 @@
       </c>
     </row>
     <row r="2686" spans="1:16">
+      <c r="B2686" s="1">
+        <v>0.58958333333333335</v>
+      </c>
       <c r="C2686" s="3" t="s">
         <v>58</v>
       </c>
@@ -69783,6 +70140,18 @@
       <c r="H2686">
         <v>0</v>
       </c>
+      <c r="L2686">
+        <v>10.9</v>
+      </c>
+      <c r="M2686">
+        <v>102.5</v>
+      </c>
+      <c r="N2686">
+        <v>1.41</v>
+      </c>
+      <c r="O2686">
+        <v>0.05</v>
+      </c>
     </row>
     <row r="2687" spans="1:16">
       <c r="D2687">
@@ -69812,7 +70181,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2689" spans="3:8">
+    <row r="2689" spans="2:15">
+      <c r="B2689" s="1">
+        <v>0.61319444444444449</v>
+      </c>
       <c r="C2689" s="3" t="s">
         <v>29</v>
       </c>
@@ -69828,8 +70200,20 @@
       <c r="H2689">
         <v>0</v>
       </c>
-    </row>
-    <row r="2690" spans="3:8">
+      <c r="L2689">
+        <v>10.7</v>
+      </c>
+      <c r="M2689">
+        <v>103.6</v>
+      </c>
+      <c r="N2689">
+        <v>4.34</v>
+      </c>
+      <c r="O2689">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="2690" spans="2:15">
       <c r="D2690">
         <v>2</v>
       </c>
@@ -69843,7 +70227,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2691" spans="3:8">
+    <row r="2691" spans="2:15">
       <c r="D2691">
         <v>3</v>
       </c>
@@ -69857,7 +70241,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2692" spans="3:8">
+    <row r="2692" spans="2:15">
+      <c r="B2692" s="1">
+        <v>0.63194444444444442</v>
+      </c>
       <c r="C2692" s="3" t="s">
         <v>30</v>
       </c>
@@ -69873,8 +70260,20 @@
       <c r="H2692">
         <v>0.28000000000000003</v>
       </c>
-    </row>
-    <row r="2693" spans="3:8">
+      <c r="L2692">
+        <v>11</v>
+      </c>
+      <c r="M2692">
+        <v>104.3</v>
+      </c>
+      <c r="N2692">
+        <v>2.39</v>
+      </c>
+      <c r="O2692">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="2693" spans="2:15">
       <c r="D2693">
         <v>2</v>
       </c>
@@ -69888,7 +70287,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2694" spans="3:8">
+    <row r="2694" spans="2:15">
       <c r="D2694">
         <v>3</v>
       </c>
@@ -69902,7 +70301,10 @@
         <v>13.18</v>
       </c>
     </row>
-    <row r="2695" spans="3:8">
+    <row r="2695" spans="2:15">
+      <c r="B2695" s="1">
+        <v>0.64513888888888893</v>
+      </c>
       <c r="C2695" s="3" t="s">
         <v>31</v>
       </c>
@@ -69918,8 +70320,20 @@
       <c r="H2695">
         <v>0</v>
       </c>
-    </row>
-    <row r="2696" spans="3:8">
+      <c r="L2695">
+        <v>12</v>
+      </c>
+      <c r="M2695">
+        <v>101.6</v>
+      </c>
+      <c r="N2695">
+        <v>1.49</v>
+      </c>
+      <c r="O2695">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="2696" spans="2:15">
       <c r="D2696">
         <v>2</v>
       </c>
@@ -69933,7 +70347,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2697" spans="3:8">
+    <row r="2697" spans="2:15">
       <c r="D2697">
         <v>3</v>
       </c>
@@ -69947,7 +70361,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2698" spans="3:8">
+    <row r="2698" spans="2:15">
+      <c r="B2698" s="1">
+        <v>0.65833333333333333</v>
+      </c>
       <c r="C2698" s="3" t="s">
         <v>32</v>
       </c>
@@ -69963,8 +70380,20 @@
       <c r="H2698">
         <v>0</v>
       </c>
-    </row>
-    <row r="2699" spans="3:8">
+      <c r="L2698">
+        <v>11.6</v>
+      </c>
+      <c r="M2698">
+        <v>105.6</v>
+      </c>
+      <c r="N2698">
+        <v>1.98</v>
+      </c>
+      <c r="O2698">
+        <v>0.19</v>
+      </c>
+    </row>
+    <row r="2699" spans="2:15">
       <c r="D2699">
         <v>2</v>
       </c>
@@ -69978,7 +70407,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2700" spans="3:8">
+    <row r="2700" spans="2:15">
       <c r="D2700">
         <v>3</v>
       </c>
@@ -69992,7 +70421,10 @@
         <v>0.28000000000000003</v>
       </c>
     </row>
-    <row r="2701" spans="3:8">
+    <row r="2701" spans="2:15">
+      <c r="B2701" s="1">
+        <v>0.67222222222222228</v>
+      </c>
       <c r="C2701" s="3" t="s">
         <v>41</v>
       </c>
@@ -70008,8 +70440,20 @@
       <c r="H2701">
         <v>0.04</v>
       </c>
-    </row>
-    <row r="2702" spans="3:8">
+      <c r="L2701">
+        <v>12.6</v>
+      </c>
+      <c r="M2701">
+        <v>105.8</v>
+      </c>
+      <c r="N2701">
+        <v>6.63</v>
+      </c>
+      <c r="O2701">
+        <v>0.92</v>
+      </c>
+    </row>
+    <row r="2702" spans="2:15">
       <c r="D2702">
         <v>2</v>
       </c>
@@ -70023,7 +70467,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="2703" spans="3:8">
+    <row r="2703" spans="2:15">
       <c r="D2703">
         <v>3</v>
       </c>
@@ -70037,7 +70481,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="2704" spans="3:8">
+    <row r="2704" spans="2:15">
       <c r="C2704" s="3" t="s">
         <v>34</v>
       </c>
@@ -70053,8 +70497,20 @@
       <c r="H2704">
         <v>0</v>
       </c>
-    </row>
-    <row r="2705" spans="3:8">
+      <c r="L2704">
+        <v>14.3</v>
+      </c>
+      <c r="M2704">
+        <v>106.6</v>
+      </c>
+      <c r="N2704">
+        <v>9.81</v>
+      </c>
+      <c r="O2704">
+        <v>0.82</v>
+      </c>
+    </row>
+    <row r="2705" spans="1:15">
       <c r="C2705" s="3"/>
       <c r="D2705">
         <v>2</v>
@@ -70069,7 +70525,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2706" spans="3:8">
+    <row r="2706" spans="1:15">
       <c r="D2706">
         <v>3</v>
       </c>
@@ -70083,8 +70539,1225 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2707" spans="3:8" s="19" customFormat="1">
+    <row r="2707" spans="1:15" s="19" customFormat="1">
       <c r="E2707" s="36"/>
+    </row>
+    <row r="2708" spans="1:15">
+      <c r="A2708" t="s">
+        <v>391</v>
+      </c>
+      <c r="B2708" s="1">
+        <v>0.55833333333333335</v>
+      </c>
+      <c r="C2708" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2708">
+        <v>1</v>
+      </c>
+      <c r="E2708" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F2708">
+        <v>0.1</v>
+      </c>
+      <c r="G2708">
+        <v>0</v>
+      </c>
+      <c r="H2708">
+        <v>0</v>
+      </c>
+      <c r="L2708">
+        <v>12.5</v>
+      </c>
+      <c r="M2708">
+        <v>97.5</v>
+      </c>
+      <c r="N2708">
+        <v>0.98</v>
+      </c>
+      <c r="O2708">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="2709" spans="1:15">
+      <c r="D2709">
+        <v>2</v>
+      </c>
+      <c r="F2709">
+        <v>0.1</v>
+      </c>
+      <c r="G2709">
+        <v>0</v>
+      </c>
+      <c r="H2709">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2710" spans="1:15">
+      <c r="D2710">
+        <v>3</v>
+      </c>
+      <c r="F2710">
+        <v>0.1</v>
+      </c>
+      <c r="G2710">
+        <v>0</v>
+      </c>
+      <c r="H2710">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2711" spans="1:15">
+      <c r="B2711" s="1">
+        <v>0.57013888888888886</v>
+      </c>
+      <c r="C2711" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2711">
+        <v>1</v>
+      </c>
+      <c r="F2711">
+        <v>0.1</v>
+      </c>
+      <c r="G2711">
+        <v>0</v>
+      </c>
+      <c r="H2711">
+        <v>0</v>
+      </c>
+      <c r="L2711">
+        <v>11.7</v>
+      </c>
+      <c r="M2711">
+        <v>95.2</v>
+      </c>
+      <c r="N2711">
+        <v>3.69</v>
+      </c>
+      <c r="O2711">
+        <v>0.14000000000000001</v>
+      </c>
+    </row>
+    <row r="2712" spans="1:15">
+      <c r="D2712">
+        <v>2</v>
+      </c>
+      <c r="F2712">
+        <v>0.1</v>
+      </c>
+      <c r="G2712">
+        <v>0</v>
+      </c>
+      <c r="H2712">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2713" spans="1:15">
+      <c r="D2713">
+        <v>3</v>
+      </c>
+      <c r="F2713">
+        <v>0.1</v>
+      </c>
+      <c r="G2713">
+        <v>0</v>
+      </c>
+      <c r="H2713">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2714" spans="1:15">
+      <c r="B2714" s="1">
+        <v>0.57986111111111116</v>
+      </c>
+      <c r="C2714" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D2714">
+        <v>1</v>
+      </c>
+      <c r="F2714">
+        <v>0.1</v>
+      </c>
+      <c r="G2714">
+        <v>0</v>
+      </c>
+      <c r="H2714">
+        <v>0</v>
+      </c>
+      <c r="L2714">
+        <v>11.1</v>
+      </c>
+      <c r="M2714">
+        <v>100.1</v>
+      </c>
+      <c r="N2714">
+        <v>0.76</v>
+      </c>
+      <c r="O2714">
+        <v>0.44</v>
+      </c>
+    </row>
+    <row r="2715" spans="1:15">
+      <c r="D2715">
+        <v>2</v>
+      </c>
+      <c r="F2715">
+        <v>0.1</v>
+      </c>
+      <c r="G2715">
+        <v>0</v>
+      </c>
+      <c r="H2715">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2716" spans="1:15">
+      <c r="D2716">
+        <v>3</v>
+      </c>
+      <c r="F2716">
+        <v>0.1</v>
+      </c>
+      <c r="G2716">
+        <v>0</v>
+      </c>
+      <c r="H2716">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2717" spans="1:15">
+      <c r="B2717" s="1">
+        <v>0.59097222222222223</v>
+      </c>
+      <c r="C2717" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D2717">
+        <v>1</v>
+      </c>
+      <c r="F2717">
+        <v>0.1</v>
+      </c>
+      <c r="G2717">
+        <v>0</v>
+      </c>
+      <c r="H2717">
+        <v>0</v>
+      </c>
+      <c r="L2717">
+        <v>11.5</v>
+      </c>
+      <c r="M2717">
+        <v>101.3</v>
+      </c>
+      <c r="N2717">
+        <v>0.64</v>
+      </c>
+      <c r="O2717">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="2718" spans="1:15">
+      <c r="D2718">
+        <v>2</v>
+      </c>
+      <c r="F2718">
+        <v>0.1</v>
+      </c>
+      <c r="G2718">
+        <v>0</v>
+      </c>
+      <c r="H2718">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2719" spans="1:15">
+      <c r="D2719">
+        <v>3</v>
+      </c>
+      <c r="F2719">
+        <v>0.1</v>
+      </c>
+      <c r="G2719">
+        <v>0</v>
+      </c>
+      <c r="H2719">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2720" spans="1:15">
+      <c r="B2720" s="1">
+        <v>0.60277777777777775</v>
+      </c>
+      <c r="C2720" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D2720">
+        <v>1</v>
+      </c>
+      <c r="F2720">
+        <v>0.1</v>
+      </c>
+      <c r="G2720">
+        <v>0</v>
+      </c>
+      <c r="H2720">
+        <v>0</v>
+      </c>
+      <c r="L2720">
+        <v>11.4</v>
+      </c>
+      <c r="M2720">
+        <v>108.2</v>
+      </c>
+      <c r="N2720">
+        <v>0.68</v>
+      </c>
+      <c r="O2720">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="2721" spans="2:15">
+      <c r="D2721">
+        <v>2</v>
+      </c>
+      <c r="F2721">
+        <v>0.1</v>
+      </c>
+      <c r="G2721">
+        <v>0</v>
+      </c>
+      <c r="H2721">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2722" spans="2:15">
+      <c r="D2722">
+        <v>3</v>
+      </c>
+      <c r="F2722">
+        <v>0.1</v>
+      </c>
+      <c r="G2722">
+        <v>0</v>
+      </c>
+      <c r="H2722">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2723" spans="2:15">
+      <c r="B2723" s="1">
+        <v>0.60833333333333328</v>
+      </c>
+      <c r="C2723" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D2723">
+        <v>1</v>
+      </c>
+      <c r="F2723">
+        <v>0.1</v>
+      </c>
+      <c r="G2723">
+        <v>0</v>
+      </c>
+      <c r="H2723">
+        <v>0</v>
+      </c>
+      <c r="L2723">
+        <v>11.3</v>
+      </c>
+      <c r="M2723">
+        <v>103.9</v>
+      </c>
+      <c r="N2723">
+        <v>0.67</v>
+      </c>
+      <c r="O2723">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="2724" spans="2:15">
+      <c r="D2724">
+        <v>2</v>
+      </c>
+      <c r="F2724">
+        <v>0.1</v>
+      </c>
+      <c r="G2724">
+        <v>0</v>
+      </c>
+      <c r="H2724">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2725" spans="2:15">
+      <c r="D2725">
+        <v>3</v>
+      </c>
+      <c r="F2725">
+        <v>0.1</v>
+      </c>
+      <c r="G2725">
+        <v>0</v>
+      </c>
+      <c r="H2725">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2726" spans="2:15">
+      <c r="B2726" s="1">
+        <v>0.61805555555555558</v>
+      </c>
+      <c r="C2726" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D2726">
+        <v>1</v>
+      </c>
+      <c r="F2726">
+        <v>0.1</v>
+      </c>
+      <c r="G2726">
+        <v>0</v>
+      </c>
+      <c r="H2726">
+        <v>0</v>
+      </c>
+      <c r="L2726">
+        <v>12.9</v>
+      </c>
+      <c r="M2726">
+        <v>100.4</v>
+      </c>
+      <c r="N2726">
+        <v>0.23</v>
+      </c>
+      <c r="O2726">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="2727" spans="2:15">
+      <c r="D2727">
+        <v>2</v>
+      </c>
+      <c r="F2727">
+        <v>0.1</v>
+      </c>
+      <c r="G2727">
+        <v>0</v>
+      </c>
+      <c r="H2727">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2728" spans="2:15">
+      <c r="D2728">
+        <v>3</v>
+      </c>
+      <c r="F2728">
+        <v>0.1</v>
+      </c>
+      <c r="G2728">
+        <v>0</v>
+      </c>
+      <c r="H2728">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2729" spans="2:15">
+      <c r="B2729" s="1">
+        <v>0.63402777777777775</v>
+      </c>
+      <c r="C2729" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D2729">
+        <v>1</v>
+      </c>
+      <c r="F2729">
+        <v>0.1</v>
+      </c>
+      <c r="G2729">
+        <v>0</v>
+      </c>
+      <c r="H2729">
+        <v>0</v>
+      </c>
+      <c r="L2729">
+        <v>11.6</v>
+      </c>
+      <c r="M2729">
+        <v>96.7</v>
+      </c>
+      <c r="N2729">
+        <v>1.28</v>
+      </c>
+      <c r="O2729">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="2730" spans="2:15">
+      <c r="D2730">
+        <v>2</v>
+      </c>
+      <c r="F2730">
+        <v>0.1</v>
+      </c>
+      <c r="G2730">
+        <v>0</v>
+      </c>
+      <c r="H2730">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2731" spans="2:15">
+      <c r="D2731">
+        <v>3</v>
+      </c>
+      <c r="F2731">
+        <v>0.1</v>
+      </c>
+      <c r="G2731">
+        <v>0</v>
+      </c>
+      <c r="H2731">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2732" spans="2:15">
+      <c r="B2732" s="1">
+        <v>0.65</v>
+      </c>
+      <c r="C2732" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="D2732">
+        <v>1</v>
+      </c>
+      <c r="F2732">
+        <v>0.1</v>
+      </c>
+      <c r="G2732">
+        <v>10.78</v>
+      </c>
+      <c r="H2732">
+        <v>0</v>
+      </c>
+      <c r="L2732">
+        <v>12.6</v>
+      </c>
+      <c r="M2732">
+        <v>101.4</v>
+      </c>
+      <c r="N2732">
+        <v>3.71</v>
+      </c>
+      <c r="O2732">
+        <v>2.68</v>
+      </c>
+    </row>
+    <row r="2733" spans="2:15">
+      <c r="D2733">
+        <v>2</v>
+      </c>
+      <c r="F2733">
+        <v>0</v>
+      </c>
+      <c r="G2733">
+        <v>9.01</v>
+      </c>
+      <c r="H2733">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="2734" spans="2:15">
+      <c r="D2734">
+        <v>3</v>
+      </c>
+      <c r="F2734">
+        <v>0.1</v>
+      </c>
+      <c r="G2734">
+        <v>3.01</v>
+      </c>
+      <c r="H2734">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="2735" spans="2:15">
+      <c r="B2735" s="1">
+        <v>0.66319444444444442</v>
+      </c>
+      <c r="C2735" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="D2735">
+        <v>1</v>
+      </c>
+      <c r="F2735">
+        <v>0.1</v>
+      </c>
+      <c r="G2735">
+        <v>1.04</v>
+      </c>
+      <c r="H2735">
+        <v>0.09</v>
+      </c>
+      <c r="L2735">
+        <v>13.9</v>
+      </c>
+      <c r="M2735">
+        <v>98.9</v>
+      </c>
+      <c r="N2735">
+        <v>2.31</v>
+      </c>
+      <c r="O2735">
+        <v>1.69</v>
+      </c>
+    </row>
+    <row r="2736" spans="2:15">
+      <c r="C2736" s="3"/>
+      <c r="D2736">
+        <v>2</v>
+      </c>
+      <c r="F2736">
+        <v>0.1</v>
+      </c>
+      <c r="G2736">
+        <v>5.37</v>
+      </c>
+      <c r="H2736">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="2737" spans="1:15">
+      <c r="D2737">
+        <v>3</v>
+      </c>
+      <c r="F2737">
+        <v>0.1</v>
+      </c>
+      <c r="G2737">
+        <v>7.44</v>
+      </c>
+      <c r="H2737">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="2738" spans="1:15" s="19" customFormat="1">
+      <c r="E2738" s="36"/>
+    </row>
+    <row r="2739" spans="1:15">
+      <c r="A2739" t="s">
+        <v>392</v>
+      </c>
+      <c r="B2739" s="1">
+        <v>0.57152777777777775</v>
+      </c>
+      <c r="C2739" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2739">
+        <v>1</v>
+      </c>
+      <c r="F2739">
+        <v>0.1</v>
+      </c>
+      <c r="G2739">
+        <v>2.27</v>
+      </c>
+      <c r="H2739">
+        <v>0.04</v>
+      </c>
+      <c r="L2739">
+        <v>13.1</v>
+      </c>
+      <c r="M2739">
+        <v>96.8</v>
+      </c>
+      <c r="N2739">
+        <v>13.21</v>
+      </c>
+      <c r="O2739">
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="2740" spans="1:15">
+      <c r="D2740">
+        <v>2</v>
+      </c>
+      <c r="F2740">
+        <v>0.1</v>
+      </c>
+      <c r="G2740">
+        <v>1.73</v>
+      </c>
+      <c r="H2740">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="2741" spans="1:15">
+      <c r="D2741">
+        <v>3</v>
+      </c>
+      <c r="F2741">
+        <v>0.1</v>
+      </c>
+      <c r="G2741">
+        <v>2.81</v>
+      </c>
+      <c r="H2741">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="2742" spans="1:15">
+      <c r="B2742" s="1">
+        <v>0.55277777777777781</v>
+      </c>
+      <c r="C2742" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2742">
+        <v>1</v>
+      </c>
+      <c r="F2742">
+        <v>0.1</v>
+      </c>
+      <c r="G2742">
+        <v>1.39</v>
+      </c>
+      <c r="H2742">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="L2742">
+        <v>12.9</v>
+      </c>
+      <c r="M2742">
+        <v>95.4</v>
+      </c>
+      <c r="N2742">
+        <v>21.71</v>
+      </c>
+      <c r="O2742">
+        <v>1.48</v>
+      </c>
+    </row>
+    <row r="2743" spans="1:15">
+      <c r="D2743">
+        <v>2</v>
+      </c>
+      <c r="F2743">
+        <v>0.1</v>
+      </c>
+      <c r="G2743">
+        <v>1.04</v>
+      </c>
+      <c r="H2743">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="2744" spans="1:15">
+      <c r="D2744">
+        <v>3</v>
+      </c>
+      <c r="F2744">
+        <v>0.1</v>
+      </c>
+      <c r="G2744">
+        <v>2.27</v>
+      </c>
+      <c r="H2744">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="2745" spans="1:15">
+      <c r="B2745" s="1">
+        <v>0.53541666666666665</v>
+      </c>
+      <c r="C2745" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D2745">
+        <v>1</v>
+      </c>
+      <c r="F2745">
+        <v>19.39</v>
+      </c>
+      <c r="G2745">
+        <v>0</v>
+      </c>
+      <c r="H2745">
+        <v>0</v>
+      </c>
+      <c r="L2745">
+        <v>11.8</v>
+      </c>
+      <c r="M2745">
+        <v>93.9</v>
+      </c>
+      <c r="N2745">
+        <v>13.29</v>
+      </c>
+      <c r="O2745">
+        <v>1.1000000000000001</v>
+      </c>
+    </row>
+    <row r="2746" spans="1:15">
+      <c r="D2746">
+        <v>2</v>
+      </c>
+      <c r="F2746">
+        <v>6.25</v>
+      </c>
+      <c r="G2746">
+        <v>0</v>
+      </c>
+      <c r="H2746">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2747" spans="1:15">
+      <c r="D2747">
+        <v>3</v>
+      </c>
+      <c r="F2747">
+        <v>0.1</v>
+      </c>
+      <c r="G2747">
+        <v>1</v>
+      </c>
+      <c r="H2747">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="2748" spans="1:15">
+      <c r="B2748" s="1">
+        <v>0.52013888888888893</v>
+      </c>
+      <c r="C2748" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D2748">
+        <v>1</v>
+      </c>
+      <c r="F2748">
+        <v>6.25</v>
+      </c>
+      <c r="G2748">
+        <v>3.01</v>
+      </c>
+      <c r="H2748">
+        <v>2.0699999999999998</v>
+      </c>
+      <c r="L2748">
+        <v>12.2</v>
+      </c>
+      <c r="M2748">
+        <v>88.4</v>
+      </c>
+      <c r="N2748">
+        <v>76.72</v>
+      </c>
+      <c r="O2748">
+        <v>9.84</v>
+      </c>
+    </row>
+    <row r="2749" spans="1:15">
+      <c r="D2749">
+        <v>2</v>
+      </c>
+      <c r="F2749">
+        <v>35.82</v>
+      </c>
+      <c r="G2749">
+        <v>1.34</v>
+      </c>
+      <c r="H2749">
+        <v>26.73</v>
+      </c>
+    </row>
+    <row r="2750" spans="1:15">
+      <c r="D2750">
+        <v>3</v>
+      </c>
+      <c r="F2750">
+        <v>96.08</v>
+      </c>
+      <c r="G2750">
+        <v>4.63</v>
+      </c>
+      <c r="H2750">
+        <v>20.75</v>
+      </c>
+    </row>
+    <row r="2751" spans="1:15">
+      <c r="B2751" s="1">
+        <v>0.48888888888888887</v>
+      </c>
+      <c r="C2751" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D2751">
+        <v>1</v>
+      </c>
+      <c r="F2751">
+        <v>0.1</v>
+      </c>
+      <c r="G2751">
+        <v>0.05</v>
+      </c>
+      <c r="H2751">
+        <v>2</v>
+      </c>
+      <c r="L2751">
+        <v>12.6</v>
+      </c>
+      <c r="M2751">
+        <v>96.1</v>
+      </c>
+      <c r="N2751">
+        <v>7.11</v>
+      </c>
+      <c r="O2751">
+        <v>3.56</v>
+      </c>
+    </row>
+    <row r="2752" spans="1:15">
+      <c r="D2752">
+        <v>2</v>
+      </c>
+      <c r="F2752">
+        <v>0.1</v>
+      </c>
+      <c r="G2752">
+        <v>2.77</v>
+      </c>
+      <c r="H2752">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="2753" spans="2:15">
+      <c r="D2753">
+        <v>3</v>
+      </c>
+      <c r="F2753">
+        <v>0.1</v>
+      </c>
+      <c r="G2753">
+        <v>3.95</v>
+      </c>
+      <c r="H2753">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="2754" spans="2:15">
+      <c r="B2754" s="1">
+        <v>0.4826388888888889</v>
+      </c>
+      <c r="C2754" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D2754">
+        <v>1</v>
+      </c>
+      <c r="F2754">
+        <v>0.1</v>
+      </c>
+      <c r="G2754">
+        <v>0.05</v>
+      </c>
+      <c r="H2754">
+        <v>2</v>
+      </c>
+      <c r="L2754">
+        <v>12.2</v>
+      </c>
+      <c r="M2754">
+        <v>99.2</v>
+      </c>
+      <c r="N2754">
+        <v>0.85</v>
+      </c>
+      <c r="O2754">
+        <v>0.26</v>
+      </c>
+    </row>
+    <row r="2755" spans="2:15">
+      <c r="D2755">
+        <v>2</v>
+      </c>
+      <c r="F2755">
+        <v>7.75</v>
+      </c>
+      <c r="G2755">
+        <v>0.6</v>
+      </c>
+      <c r="H2755">
+        <v>12.91</v>
+      </c>
+    </row>
+    <row r="2756" spans="2:15">
+      <c r="D2756">
+        <v>3</v>
+      </c>
+      <c r="F2756">
+        <v>20.170000000000002</v>
+      </c>
+      <c r="G2756">
+        <v>0.75</v>
+      </c>
+      <c r="H2756">
+        <v>26.89</v>
+      </c>
+    </row>
+    <row r="2757" spans="2:15">
+      <c r="B2757" s="1">
+        <v>0.47569444444444442</v>
+      </c>
+      <c r="C2757" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D2757">
+        <v>1</v>
+      </c>
+      <c r="F2757">
+        <v>20.95</v>
+      </c>
+      <c r="G2757">
+        <v>0.8</v>
+      </c>
+      <c r="H2757">
+        <v>26.18</v>
+      </c>
+      <c r="L2757">
+        <v>12.4</v>
+      </c>
+      <c r="M2757">
+        <v>98.6</v>
+      </c>
+      <c r="N2757">
+        <v>0.71</v>
+      </c>
+      <c r="O2757">
+        <v>0.42</v>
+      </c>
+    </row>
+    <row r="2758" spans="2:15">
+      <c r="D2758">
+        <v>2</v>
+      </c>
+      <c r="F2758">
+        <v>79.650000000000006</v>
+      </c>
+      <c r="G2758">
+        <v>1.29</v>
+      </c>
+      <c r="H2758">
+        <v>61.74</v>
+      </c>
+    </row>
+    <row r="2759" spans="2:15">
+      <c r="D2759">
+        <v>3</v>
+      </c>
+      <c r="F2759">
+        <v>25.65</v>
+      </c>
+      <c r="G2759">
+        <v>1.04</v>
+      </c>
+      <c r="H2759">
+        <v>24.66</v>
+      </c>
+    </row>
+    <row r="2760" spans="2:15">
+      <c r="B2760" s="1">
+        <v>0.41041666666666665</v>
+      </c>
+      <c r="C2760" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D2760">
+        <v>1</v>
+      </c>
+      <c r="F2760">
+        <v>34.25</v>
+      </c>
+      <c r="G2760">
+        <v>0.95</v>
+      </c>
+      <c r="H2760">
+        <v>36.06</v>
+      </c>
+      <c r="L2760">
+        <v>11</v>
+      </c>
+      <c r="M2760">
+        <v>97.3</v>
+      </c>
+      <c r="N2760">
+        <v>0.92</v>
+      </c>
+      <c r="O2760">
+        <v>0.21</v>
+      </c>
+    </row>
+    <row r="2761" spans="2:15">
+      <c r="D2761">
+        <v>2</v>
+      </c>
+      <c r="F2761">
+        <v>7.75</v>
+      </c>
+      <c r="G2761">
+        <v>0.4</v>
+      </c>
+      <c r="H2761">
+        <v>19.37</v>
+      </c>
+    </row>
+    <row r="2762" spans="2:15">
+      <c r="D2762">
+        <v>3</v>
+      </c>
+      <c r="F2762">
+        <v>40.520000000000003</v>
+      </c>
+      <c r="G2762">
+        <v>1.29</v>
+      </c>
+      <c r="H2762">
+        <v>31.41</v>
+      </c>
+    </row>
+    <row r="2763" spans="2:15">
+      <c r="B2763" s="1">
+        <v>0.4548611111111111</v>
+      </c>
+      <c r="C2763" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="D2763">
+        <v>1</v>
+      </c>
+      <c r="F2763">
+        <v>0.1</v>
+      </c>
+      <c r="G2763">
+        <v>0.3</v>
+      </c>
+      <c r="H2763">
+        <v>0.33</v>
+      </c>
+      <c r="L2763">
+        <v>12.2</v>
+      </c>
+      <c r="M2763">
+        <v>98.7</v>
+      </c>
+      <c r="N2763">
+        <v>0.81</v>
+      </c>
+      <c r="O2763">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="2764" spans="2:15">
+      <c r="D2764">
+        <v>2</v>
+      </c>
+      <c r="F2764">
+        <v>36.6</v>
+      </c>
+      <c r="G2764">
+        <v>0.75</v>
+      </c>
+      <c r="H2764">
+        <v>48.8</v>
+      </c>
+    </row>
+    <row r="2765" spans="2:15">
+      <c r="D2765">
+        <v>3</v>
+      </c>
+      <c r="F2765">
+        <v>39.729999999999997</v>
+      </c>
+      <c r="G2765">
+        <v>0.85</v>
+      </c>
+      <c r="H2765">
+        <v>46.74</v>
+      </c>
+    </row>
+    <row r="2766" spans="2:15">
+      <c r="B2766" s="1">
+        <v>0.58888888888888891</v>
+      </c>
+      <c r="C2766" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="D2766">
+        <v>1</v>
+      </c>
+      <c r="F2766">
+        <v>0.1</v>
+      </c>
+      <c r="G2766">
+        <v>1.63</v>
+      </c>
+      <c r="H2766">
+        <v>0.06</v>
+      </c>
+      <c r="L2766">
+        <v>15.3</v>
+      </c>
+      <c r="M2766">
+        <v>97.6</v>
+      </c>
+      <c r="N2766">
+        <v>0.84</v>
+      </c>
+      <c r="O2766">
+        <v>0.66</v>
+      </c>
+    </row>
+    <row r="2767" spans="2:15">
+      <c r="C2767" s="3"/>
+      <c r="D2767">
+        <v>2</v>
+      </c>
+      <c r="F2767">
+        <v>0.1</v>
+      </c>
+      <c r="G2767">
+        <v>1.0900000000000001</v>
+      </c>
+      <c r="H2767">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="2768" spans="2:15">
+      <c r="D2768">
+        <v>3</v>
+      </c>
+      <c r="F2768">
+        <v>0.1</v>
+      </c>
+      <c r="G2768">
+        <v>1.73</v>
+      </c>
+      <c r="H2768">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="2769" spans="5:5" s="19" customFormat="1">
+      <c r="E2769" s="36"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>